<commit_message>
include the updated code
</commit_message>
<xml_diff>
--- a/feature_extraction_code/extracted_features/extracted_features.xlsx
+++ b/feature_extraction_code/extracted_features/extracted_features.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CG76"/>
+  <dimension ref="A1:CW76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -842,6 +842,86 @@
           <t>bbox_elongation</t>
         </is>
       </c>
+      <c r="CH1" t="inlineStr">
+        <is>
+          <t>surface_coverage_ratio</t>
+        </is>
+      </c>
+      <c r="CI1" t="inlineStr">
+        <is>
+          <t>pixel_std_x</t>
+        </is>
+      </c>
+      <c r="CJ1" t="inlineStr">
+        <is>
+          <t>pixel_std_y</t>
+        </is>
+      </c>
+      <c r="CK1" t="inlineStr">
+        <is>
+          <t>mean_distance_center</t>
+        </is>
+      </c>
+      <c r="CL1" t="inlineStr">
+        <is>
+          <t>left_right_balance</t>
+        </is>
+      </c>
+      <c r="CM1" t="inlineStr">
+        <is>
+          <t>top_bottom_balance</t>
+        </is>
+      </c>
+      <c r="CN1" t="inlineStr">
+        <is>
+          <t>colors_used_count</t>
+        </is>
+      </c>
+      <c r="CO1" t="inlineStr">
+        <is>
+          <t>mean_hue</t>
+        </is>
+      </c>
+      <c r="CP1" t="inlineStr">
+        <is>
+          <t>std_hue</t>
+        </is>
+      </c>
+      <c r="CQ1" t="inlineStr">
+        <is>
+          <t>mean_saturation</t>
+        </is>
+      </c>
+      <c r="CR1" t="inlineStr">
+        <is>
+          <t>std_saturation</t>
+        </is>
+      </c>
+      <c r="CS1" t="inlineStr">
+        <is>
+          <t>mean_brightness</t>
+        </is>
+      </c>
+      <c r="CT1" t="inlineStr">
+        <is>
+          <t>std_brightness</t>
+        </is>
+      </c>
+      <c r="CU1" t="inlineStr">
+        <is>
+          <t>black_ratio</t>
+        </is>
+      </c>
+      <c r="CV1" t="inlineStr">
+        <is>
+          <t>warm_cool_ratio</t>
+        </is>
+      </c>
+      <c r="CW1" t="inlineStr">
+        <is>
+          <t>brightness_range</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1109,6 +1189,54 @@
       <c r="CG2" t="n">
         <v>0.3307638402242466</v>
       </c>
+      <c r="CH2" t="n">
+        <v>0.03929259505175735</v>
+      </c>
+      <c r="CI2" t="n">
+        <v>0.3102734262938263</v>
+      </c>
+      <c r="CJ2" t="n">
+        <v>0.2525624650807408</v>
+      </c>
+      <c r="CK2" t="n">
+        <v>2650310.186795299</v>
+      </c>
+      <c r="CL2" t="n">
+        <v>-0.1212100225771154</v>
+      </c>
+      <c r="CM2" t="n">
+        <v>0.4641328587060404</v>
+      </c>
+      <c r="CN2" t="n">
+        <v>6</v>
+      </c>
+      <c r="CO2" t="n">
+        <v>17.59228806488468</v>
+      </c>
+      <c r="CP2" t="n">
+        <v>15.59915534856525</v>
+      </c>
+      <c r="CQ2" t="n">
+        <v>0.327010817624001</v>
+      </c>
+      <c r="CR2" t="n">
+        <v>0.4512866675201521</v>
+      </c>
+      <c r="CS2" t="n">
+        <v>0.7546085642035532</v>
+      </c>
+      <c r="CT2" t="n">
+        <v>0.2384087041649999</v>
+      </c>
+      <c r="CU2" t="n">
+        <v>0.03313157056387384</v>
+      </c>
+      <c r="CV2" t="n">
+        <v>2.448956193568791</v>
+      </c>
+      <c r="CW2" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1376,6 +1504,54 @@
       <c r="CG3" t="n">
         <v>0.1892857142857142</v>
       </c>
+      <c r="CH3" t="n">
+        <v>0.01033078991194174</v>
+      </c>
+      <c r="CI3" t="n">
+        <v>0.05911754796233108</v>
+      </c>
+      <c r="CJ3" t="n">
+        <v>0.1120926562788098</v>
+      </c>
+      <c r="CK3" t="n">
+        <v>2052848.051058928</v>
+      </c>
+      <c r="CL3" t="n">
+        <v>1</v>
+      </c>
+      <c r="CM3" t="n">
+        <v>0.3207248972710989</v>
+      </c>
+      <c r="CN3" t="n">
+        <v>1</v>
+      </c>
+      <c r="CO3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU3" t="n">
+        <v>1</v>
+      </c>
+      <c r="CV3" t="n">
+        <v>1898200000000</v>
+      </c>
+      <c r="CW3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1643,6 +1819,54 @@
       <c r="CG4" t="n">
         <v>0.482998454404946</v>
       </c>
+      <c r="CH4" t="n">
+        <v>0.01814881736347705</v>
+      </c>
+      <c r="CI4" t="n">
+        <v>0.2832023075425686</v>
+      </c>
+      <c r="CJ4" t="n">
+        <v>0.2064693218334176</v>
+      </c>
+      <c r="CK4" t="n">
+        <v>2351126.606939354</v>
+      </c>
+      <c r="CL4" t="n">
+        <v>0.243350226407173</v>
+      </c>
+      <c r="CM4" t="n">
+        <v>-0.6545416379284493</v>
+      </c>
+      <c r="CN4" t="n">
+        <v>2</v>
+      </c>
+      <c r="CO4" t="n">
+        <v>22.35468672368005</v>
+      </c>
+      <c r="CP4" t="n">
+        <v>26.86073561761302</v>
+      </c>
+      <c r="CQ4" t="n">
+        <v>0.2773262962185504</v>
+      </c>
+      <c r="CR4" t="n">
+        <v>0.4476789269602169</v>
+      </c>
+      <c r="CS4" t="n">
+        <v>0.2773262962185504</v>
+      </c>
+      <c r="CT4" t="n">
+        <v>0.4476789269602169</v>
+      </c>
+      <c r="CU4" t="n">
+        <v>0.7226737037814496</v>
+      </c>
+      <c r="CV4" t="n">
+        <v>2.605860726640781</v>
+      </c>
+      <c r="CW4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1910,6 +2134,54 @@
       <c r="CG5" t="n">
         <v>0.137792103142627</v>
       </c>
+      <c r="CH5" t="n">
+        <v>0.05311632615297537</v>
+      </c>
+      <c r="CI5" t="n">
+        <v>0.0861083548447425</v>
+      </c>
+      <c r="CJ5" t="n">
+        <v>0.09864909313642602</v>
+      </c>
+      <c r="CK5" t="n">
+        <v>1237068.337623353</v>
+      </c>
+      <c r="CL5" t="n">
+        <v>0.3340778917384756</v>
+      </c>
+      <c r="CM5" t="n">
+        <v>1</v>
+      </c>
+      <c r="CN5" t="n">
+        <v>5</v>
+      </c>
+      <c r="CO5" t="n">
+        <v>5.487159039910003</v>
+      </c>
+      <c r="CP5" t="n">
+        <v>9.743677627580086</v>
+      </c>
+      <c r="CQ5" t="n">
+        <v>0.1191204647683843</v>
+      </c>
+      <c r="CR5" t="n">
+        <v>0.2475915380773528</v>
+      </c>
+      <c r="CS5" t="n">
+        <v>0.2050903203991926</v>
+      </c>
+      <c r="CT5" t="n">
+        <v>0.3921568732227363</v>
+      </c>
+      <c r="CU5" t="n">
+        <v>0.7718065104460178</v>
+      </c>
+      <c r="CV5" t="n">
+        <v>88.53853210927947</v>
+      </c>
+      <c r="CW5" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2177,6 +2449,54 @@
       <c r="CG6" t="n">
         <v>0.2213438735177866</v>
       </c>
+      <c r="CH6" t="n">
+        <v>0.04203611585810538</v>
+      </c>
+      <c r="CI6" t="n">
+        <v>0.1202655934749524</v>
+      </c>
+      <c r="CJ6" t="n">
+        <v>0.1239894095300643</v>
+      </c>
+      <c r="CK6" t="n">
+        <v>1355655.782246023</v>
+      </c>
+      <c r="CL6" t="n">
+        <v>0.4570548175768404</v>
+      </c>
+      <c r="CM6" t="n">
+        <v>0.4695357207592118</v>
+      </c>
+      <c r="CN6" t="n">
+        <v>4</v>
+      </c>
+      <c r="CO6" t="n">
+        <v>179.5381847460876</v>
+      </c>
+      <c r="CP6" t="n">
+        <v>46.98676817276458</v>
+      </c>
+      <c r="CQ6" t="n">
+        <v>0.196468059763329</v>
+      </c>
+      <c r="CR6" t="n">
+        <v>0.3408945208956088</v>
+      </c>
+      <c r="CS6" t="n">
+        <v>0.235542090680753</v>
+      </c>
+      <c r="CT6" t="n">
+        <v>0.3924695398192671</v>
+      </c>
+      <c r="CU6" t="n">
+        <v>0.6993837230378829</v>
+      </c>
+      <c r="CV6" t="n">
+        <v>6.871789645325242</v>
+      </c>
+      <c r="CW6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2444,6 +2764,54 @@
       <c r="CG7" t="n">
         <v>0.07715430861723449</v>
       </c>
+      <c r="CH7" t="n">
+        <v>0.02790597685885644</v>
+      </c>
+      <c r="CI7" t="n">
+        <v>0.1343648506908806</v>
+      </c>
+      <c r="CJ7" t="n">
+        <v>0.2134736285983381</v>
+      </c>
+      <c r="CK7" t="n">
+        <v>1935756.438454655</v>
+      </c>
+      <c r="CL7" t="n">
+        <v>-0.8359824475865432</v>
+      </c>
+      <c r="CM7" t="n">
+        <v>-0.5403217942467089</v>
+      </c>
+      <c r="CN7" t="n">
+        <v>3</v>
+      </c>
+      <c r="CO7" t="n">
+        <v>37.06063098696232</v>
+      </c>
+      <c r="CP7" t="n">
+        <v>38.22207281769195</v>
+      </c>
+      <c r="CQ7" t="n">
+        <v>0.6642808386153096</v>
+      </c>
+      <c r="CR7" t="n">
+        <v>0.4722412583244401</v>
+      </c>
+      <c r="CS7" t="n">
+        <v>0.6642808386153096</v>
+      </c>
+      <c r="CT7" t="n">
+        <v>0.4722412583244401</v>
+      </c>
+      <c r="CU7" t="n">
+        <v>0.3357191613846904</v>
+      </c>
+      <c r="CV7" t="n">
+        <v>0.505387393206158</v>
+      </c>
+      <c r="CW7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2711,6 +3079,54 @@
       <c r="CG8" t="n">
         <v>0.326817826426896</v>
       </c>
+      <c r="CH8" t="n">
+        <v>0.2226442511782826</v>
+      </c>
+      <c r="CI8" t="n">
+        <v>0.2356236364016911</v>
+      </c>
+      <c r="CJ8" t="n">
+        <v>0.2591030460671493</v>
+      </c>
+      <c r="CK8" t="n">
+        <v>2590415.506056106</v>
+      </c>
+      <c r="CL8" t="n">
+        <v>0.588037869324918</v>
+      </c>
+      <c r="CM8" t="n">
+        <v>0.3585828092038202</v>
+      </c>
+      <c r="CN8" t="n">
+        <v>3</v>
+      </c>
+      <c r="CO8" t="n">
+        <v>179.9342834498089</v>
+      </c>
+      <c r="CP8" t="n">
+        <v>5.746826431444374</v>
+      </c>
+      <c r="CQ8" t="n">
+        <v>0.0006932442903901578</v>
+      </c>
+      <c r="CR8" t="n">
+        <v>0.01663782222858222</v>
+      </c>
+      <c r="CS8" t="n">
+        <v>0.001733110725975394</v>
+      </c>
+      <c r="CT8" t="n">
+        <v>0.04159455557145555</v>
+      </c>
+      <c r="CU8" t="n">
+        <v>0.9982668892740246</v>
+      </c>
+      <c r="CV8" t="n">
+        <v>575.9971791174048</v>
+      </c>
+      <c r="CW8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2978,6 +3394,54 @@
       <c r="CG9" t="n">
         <v>0.1721419185282522</v>
       </c>
+      <c r="CH9" t="n">
+        <v>0.02481250884392246</v>
+      </c>
+      <c r="CI9" t="n">
+        <v>0.1049039839531103</v>
+      </c>
+      <c r="CJ9" t="n">
+        <v>0.1023908884469174</v>
+      </c>
+      <c r="CK9" t="n">
+        <v>1607225.967508128</v>
+      </c>
+      <c r="CL9" t="n">
+        <v>0.6848062117523195</v>
+      </c>
+      <c r="CM9" t="n">
+        <v>0.9631944901405979</v>
+      </c>
+      <c r="CN9" t="n">
+        <v>3</v>
+      </c>
+      <c r="CO9" t="n">
+        <v>7.283787709839796e-16</v>
+      </c>
+      <c r="CP9" t="n">
+        <v>25.22744077054979</v>
+      </c>
+      <c r="CQ9" t="n">
+        <v>0.08595994823539733</v>
+      </c>
+      <c r="CR9" t="n">
+        <v>0.2803048974505532</v>
+      </c>
+      <c r="CS9" t="n">
+        <v>0.2274175200557729</v>
+      </c>
+      <c r="CT9" t="n">
+        <v>0.3244185159715</v>
+      </c>
+      <c r="CU9" t="n">
+        <v>0.6322300454036981</v>
+      </c>
+      <c r="CV9" t="n">
+        <v>10.63332482773505</v>
+      </c>
+      <c r="CW9" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3245,6 +3709,54 @@
       <c r="CG10" t="n">
         <v>0.3521276595744681</v>
       </c>
+      <c r="CH10" t="n">
+        <v>0.02167441303566958</v>
+      </c>
+      <c r="CI10" t="n">
+        <v>0.2041579656714611</v>
+      </c>
+      <c r="CJ10" t="n">
+        <v>0.1530763961355726</v>
+      </c>
+      <c r="CK10" t="n">
+        <v>2098726.226709077</v>
+      </c>
+      <c r="CL10" t="n">
+        <v>0.362510985561833</v>
+      </c>
+      <c r="CM10" t="n">
+        <v>0.5563590709353421</v>
+      </c>
+      <c r="CN10" t="n">
+        <v>1</v>
+      </c>
+      <c r="CO10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU10" t="n">
+        <v>1</v>
+      </c>
+      <c r="CV10" t="n">
+        <v>3982500000000</v>
+      </c>
+      <c r="CW10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3512,6 +4024,54 @@
       <c r="CG11" t="n">
         <v>0.3343999999999999</v>
       </c>
+      <c r="CH11" t="n">
+        <v>0.05657062620413406</v>
+      </c>
+      <c r="CI11" t="n">
+        <v>0.2771208364238975</v>
+      </c>
+      <c r="CJ11" t="n">
+        <v>0.1682877214633399</v>
+      </c>
+      <c r="CK11" t="n">
+        <v>2176370.682342258</v>
+      </c>
+      <c r="CL11" t="n">
+        <v>-0.01502732240437158</v>
+      </c>
+      <c r="CM11" t="n">
+        <v>0.425652274301547</v>
+      </c>
+      <c r="CN11" t="n">
+        <v>1</v>
+      </c>
+      <c r="CO11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU11" t="n">
+        <v>1</v>
+      </c>
+      <c r="CV11" t="n">
+        <v>10394400000000</v>
+      </c>
+      <c r="CW11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3779,6 +4339,54 @@
       <c r="CG12" t="n">
         <v>0.1470113085621971</v>
       </c>
+      <c r="CH12" t="n">
+        <v>0.02437548301422647</v>
+      </c>
+      <c r="CI12" t="n">
+        <v>0.1242368364063842</v>
+      </c>
+      <c r="CJ12" t="n">
+        <v>0.1588698860530357</v>
+      </c>
+      <c r="CK12" t="n">
+        <v>1134943.481283615</v>
+      </c>
+      <c r="CL12" t="n">
+        <v>0.1564704831651335</v>
+      </c>
+      <c r="CM12" t="n">
+        <v>0.4362329195320175</v>
+      </c>
+      <c r="CN12" t="n">
+        <v>3</v>
+      </c>
+      <c r="CO12" t="n">
+        <v>163.4504460210726</v>
+      </c>
+      <c r="CP12" t="n">
+        <v>68.3210050792399</v>
+      </c>
+      <c r="CQ12" t="n">
+        <v>0.1215236223988568</v>
+      </c>
+      <c r="CR12" t="n">
+        <v>0.1899791067424237</v>
+      </c>
+      <c r="CS12" t="n">
+        <v>0.2959319460569796</v>
+      </c>
+      <c r="CT12" t="n">
+        <v>0.4554733671949326</v>
+      </c>
+      <c r="CU12" t="n">
+        <v>0.701817451102974</v>
+      </c>
+      <c r="CV12" t="n">
+        <v>2.353650318231109</v>
+      </c>
+      <c r="CW12" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4046,6 +4654,54 @@
       <c r="CG13" t="n">
         <v>0.3324070857936784</v>
       </c>
+      <c r="CH13" t="n">
+        <v>0.06801711094904812</v>
+      </c>
+      <c r="CI13" t="n">
+        <v>0.2300637392115803</v>
+      </c>
+      <c r="CJ13" t="n">
+        <v>0.2863195105989899</v>
+      </c>
+      <c r="CK13" t="n">
+        <v>2004868.346421772</v>
+      </c>
+      <c r="CL13" t="n">
+        <v>0.1448438100115222</v>
+      </c>
+      <c r="CM13" t="n">
+        <v>0.01945973626936372</v>
+      </c>
+      <c r="CN13" t="n">
+        <v>5</v>
+      </c>
+      <c r="CO13" t="n">
+        <v>6.94415239713976</v>
+      </c>
+      <c r="CP13" t="n">
+        <v>37.22366174637347</v>
+      </c>
+      <c r="CQ13" t="n">
+        <v>0.3473786967097683</v>
+      </c>
+      <c r="CR13" t="n">
+        <v>0.4761373097983303</v>
+      </c>
+      <c r="CS13" t="n">
+        <v>0.3473786967097683</v>
+      </c>
+      <c r="CT13" t="n">
+        <v>0.4761373097983303</v>
+      </c>
+      <c r="CU13" t="n">
+        <v>0.6526213032902317</v>
+      </c>
+      <c r="CV13" t="n">
+        <v>3.70701668486923</v>
+      </c>
+      <c r="CW13" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4313,6 +4969,54 @@
       <c r="CG14" t="n">
         <v>0.1497730711043873</v>
       </c>
+      <c r="CH14" t="n">
+        <v>0.05418412774433717</v>
+      </c>
+      <c r="CI14" t="n">
+        <v>0.08830929323781604</v>
+      </c>
+      <c r="CJ14" t="n">
+        <v>0.1193500714343509</v>
+      </c>
+      <c r="CK14" t="n">
+        <v>832426.153825074</v>
+      </c>
+      <c r="CL14" t="n">
+        <v>0.1526431563193684</v>
+      </c>
+      <c r="CM14" t="n">
+        <v>-0.4224329292178507</v>
+      </c>
+      <c r="CN14" t="n">
+        <v>4</v>
+      </c>
+      <c r="CO14" t="n">
+        <v>0.2866906018414734</v>
+      </c>
+      <c r="CP14" t="n">
+        <v>1.49204332359876</v>
+      </c>
+      <c r="CQ14" t="n">
+        <v>0.8734720115710283</v>
+      </c>
+      <c r="CR14" t="n">
+        <v>0.33244346372442</v>
+      </c>
+      <c r="CS14" t="n">
+        <v>0.8222762382105083</v>
+      </c>
+      <c r="CT14" t="n">
+        <v>0.354485143469618</v>
+      </c>
+      <c r="CU14" t="n">
+        <v>0.1265279884289718</v>
+      </c>
+      <c r="CV14" t="n">
+        <v>9955900000000</v>
+      </c>
+      <c r="CW14" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4580,6 +5284,54 @@
       <c r="CG15" t="n">
         <v>0.4435695538057742</v>
       </c>
+      <c r="CH15" t="n">
+        <v>0.0244783446354127</v>
+      </c>
+      <c r="CI15" t="n">
+        <v>0.1102066937297697</v>
+      </c>
+      <c r="CJ15" t="n">
+        <v>0.1378375378054231</v>
+      </c>
+      <c r="CK15" t="n">
+        <v>1378979.782449926</v>
+      </c>
+      <c r="CL15" t="n">
+        <v>0.6550681459412588</v>
+      </c>
+      <c r="CM15" t="n">
+        <v>0.921915645774507</v>
+      </c>
+      <c r="CN15" t="n">
+        <v>6</v>
+      </c>
+      <c r="CO15" t="n">
+        <v>15.46977360229429</v>
+      </c>
+      <c r="CP15" t="n">
+        <v>20.74855196554084</v>
+      </c>
+      <c r="CQ15" t="n">
+        <v>0.401872067945839</v>
+      </c>
+      <c r="CR15" t="n">
+        <v>0.4902763597714803</v>
+      </c>
+      <c r="CS15" t="n">
+        <v>0.2656157591657958</v>
+      </c>
+      <c r="CT15" t="n">
+        <v>0.3749153292899032</v>
+      </c>
+      <c r="CU15" t="n">
+        <v>0.598127932054161</v>
+      </c>
+      <c r="CV15" t="n">
+        <v>3.243513539010054</v>
+      </c>
+      <c r="CW15" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4847,6 +5599,54 @@
       <c r="CG16" t="n">
         <v>0.3161609033168666</v>
       </c>
+      <c r="CH16" t="n">
+        <v>0.03057003842344156</v>
+      </c>
+      <c r="CI16" t="n">
+        <v>0.2249242198543437</v>
+      </c>
+      <c r="CJ16" t="n">
+        <v>0.2455991384534955</v>
+      </c>
+      <c r="CK16" t="n">
+        <v>1907524.873736256</v>
+      </c>
+      <c r="CL16" t="n">
+        <v>-0.008901548869503293</v>
+      </c>
+      <c r="CM16" t="n">
+        <v>-0.09147231618301585</v>
+      </c>
+      <c r="CN16" t="n">
+        <v>3</v>
+      </c>
+      <c r="CO16" t="n">
+        <v>0.2896104314711189</v>
+      </c>
+      <c r="CP16" t="n">
+        <v>4.55072565721179</v>
+      </c>
+      <c r="CQ16" t="n">
+        <v>0.002314402706070856</v>
+      </c>
+      <c r="CR16" t="n">
+        <v>0.0303381710480786</v>
+      </c>
+      <c r="CS16" t="n">
+        <v>0.04936017063047402</v>
+      </c>
+      <c r="CT16" t="n">
+        <v>0.15881467750226</v>
+      </c>
+      <c r="CU16" t="n">
+        <v>0.9074060886594267</v>
+      </c>
+      <c r="CV16" t="n">
+        <v>171.8307692254821</v>
+      </c>
+      <c r="CW16" t="n">
+        <v>0.5019607843137255</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5114,6 +5914,54 @@
       <c r="CG17" t="n">
         <v>0.436377245508982</v>
       </c>
+      <c r="CH17" t="n">
+        <v>0.034314963372555</v>
+      </c>
+      <c r="CI17" t="n">
+        <v>0.263614494689898</v>
+      </c>
+      <c r="CJ17" t="n">
+        <v>0.2153524406198637</v>
+      </c>
+      <c r="CK17" t="n">
+        <v>2127245.686910261</v>
+      </c>
+      <c r="CL17" t="n">
+        <v>-0.1736847948486146</v>
+      </c>
+      <c r="CM17" t="n">
+        <v>0.3535074780733057</v>
+      </c>
+      <c r="CN17" t="n">
+        <v>1</v>
+      </c>
+      <c r="CO17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU17" t="n">
+        <v>1</v>
+      </c>
+      <c r="CV17" t="n">
+        <v>6305100000000</v>
+      </c>
+      <c r="CW17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5381,6 +6229,54 @@
       <c r="CG18" t="n">
         <v>0.11340206185567</v>
       </c>
+      <c r="CH18" t="n">
+        <v>0.06489370965810756</v>
+      </c>
+      <c r="CI18" t="n">
+        <v>0.127757331464884</v>
+      </c>
+      <c r="CJ18" t="n">
+        <v>0.164362336510039</v>
+      </c>
+      <c r="CK18" t="n">
+        <v>1339401.959303711</v>
+      </c>
+      <c r="CL18" t="n">
+        <v>0.256489177017201</v>
+      </c>
+      <c r="CM18" t="n">
+        <v>0.6731215981616444</v>
+      </c>
+      <c r="CN18" t="n">
+        <v>4</v>
+      </c>
+      <c r="CO18" t="n">
+        <v>175.346878713669</v>
+      </c>
+      <c r="CP18" t="n">
+        <v>60.33319780559084</v>
+      </c>
+      <c r="CQ18" t="n">
+        <v>0.160948363343593</v>
+      </c>
+      <c r="CR18" t="n">
+        <v>0.3674833161935542</v>
+      </c>
+      <c r="CS18" t="n">
+        <v>0.5081023507803786</v>
+      </c>
+      <c r="CT18" t="n">
+        <v>0.4248570988279171</v>
+      </c>
+      <c r="CU18" t="n">
+        <v>0.4051091523604251</v>
+      </c>
+      <c r="CV18" t="n">
+        <v>414.4599302991477</v>
+      </c>
+      <c r="CW18" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5648,6 +6544,54 @@
       <c r="CG19" t="n">
         <v>0.2751842751842752</v>
       </c>
+      <c r="CH19" t="n">
+        <v>0.1265486388523038</v>
+      </c>
+      <c r="CI19" t="n">
+        <v>0.2741267097760309</v>
+      </c>
+      <c r="CJ19" t="n">
+        <v>0.2187581024006512</v>
+      </c>
+      <c r="CK19" t="n">
+        <v>2207271.258119249</v>
+      </c>
+      <c r="CL19" t="n">
+        <v>-0.1450394154556754</v>
+      </c>
+      <c r="CM19" t="n">
+        <v>0.1942732546887835</v>
+      </c>
+      <c r="CN19" t="n">
+        <v>16</v>
+      </c>
+      <c r="CO19" t="n">
+        <v>14.2126530291367</v>
+      </c>
+      <c r="CP19" t="n">
+        <v>39.44538675100659</v>
+      </c>
+      <c r="CQ19" t="n">
+        <v>0.53099349311681</v>
+      </c>
+      <c r="CR19" t="n">
+        <v>0.4463341111621849</v>
+      </c>
+      <c r="CS19" t="n">
+        <v>0.737169968343001</v>
+      </c>
+      <c r="CT19" t="n">
+        <v>0.3813471100836657</v>
+      </c>
+      <c r="CU19" t="n">
+        <v>0.096209837306417</v>
+      </c>
+      <c r="CV19" t="n">
+        <v>2.186730806128582</v>
+      </c>
+      <c r="CW19" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5915,6 +6859,54 @@
       <c r="CG20" t="n">
         <v>0.03238469087340543</v>
       </c>
+      <c r="CH20" t="n">
+        <v>0.211245659674979</v>
+      </c>
+      <c r="CI20" t="n">
+        <v>0.1558677496566251</v>
+      </c>
+      <c r="CJ20" t="n">
+        <v>0.1184960129293618</v>
+      </c>
+      <c r="CK20" t="n">
+        <v>1292169.124257389</v>
+      </c>
+      <c r="CL20" t="n">
+        <v>0.2092480426230268</v>
+      </c>
+      <c r="CM20" t="n">
+        <v>0.3486642947130855</v>
+      </c>
+      <c r="CN20" t="n">
+        <v>6</v>
+      </c>
+      <c r="CO20" t="n">
+        <v>117.051876688472</v>
+      </c>
+      <c r="CP20" t="n">
+        <v>13.17612686696879</v>
+      </c>
+      <c r="CQ20" t="n">
+        <v>0.9497870652098303</v>
+      </c>
+      <c r="CR20" t="n">
+        <v>0.2183840561257343</v>
+      </c>
+      <c r="CS20" t="n">
+        <v>0.3902148958422211</v>
+      </c>
+      <c r="CT20" t="n">
+        <v>0.08380353840526376</v>
+      </c>
+      <c r="CU20" t="n">
+        <v>0.03480382432428951</v>
+      </c>
+      <c r="CV20" t="n">
+        <v>0.0528675706686689</v>
+      </c>
+      <c r="CW20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -6182,6 +7174,54 @@
       <c r="CG21" t="n">
         <v>0.328</v>
       </c>
+      <c r="CH21" t="n">
+        <v>0.06933635205886515</v>
+      </c>
+      <c r="CI21" t="n">
+        <v>0.1959614478558205</v>
+      </c>
+      <c r="CJ21" t="n">
+        <v>0.2393334351905817</v>
+      </c>
+      <c r="CK21" t="n">
+        <v>1914468.231693324</v>
+      </c>
+      <c r="CL21" t="n">
+        <v>0.08963893249607535</v>
+      </c>
+      <c r="CM21" t="n">
+        <v>0.5165149136577708</v>
+      </c>
+      <c r="CN21" t="n">
+        <v>5</v>
+      </c>
+      <c r="CO21" t="n">
+        <v>9.967401994703975</v>
+      </c>
+      <c r="CP21" t="n">
+        <v>9.905902965612041</v>
+      </c>
+      <c r="CQ21" t="n">
+        <v>0.3624568288854003</v>
+      </c>
+      <c r="CR21" t="n">
+        <v>0.4807097628296517</v>
+      </c>
+      <c r="CS21" t="n">
+        <v>0.1629136577708007</v>
+      </c>
+      <c r="CT21" t="n">
+        <v>0.2324417719718338</v>
+      </c>
+      <c r="CU21" t="n">
+        <v>0.6319387755102041</v>
+      </c>
+      <c r="CV21" t="n">
+        <v>206.1544715413633</v>
+      </c>
+      <c r="CW21" t="n">
+        <v>0.4</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -6449,6 +7489,54 @@
       <c r="CG22" t="n">
         <v>0.2663316582914573</v>
       </c>
+      <c r="CH22" t="n">
+        <v>0.01870666477996321</v>
+      </c>
+      <c r="CI22" t="n">
+        <v>0.1132267924192417</v>
+      </c>
+      <c r="CJ22" t="n">
+        <v>0.1398091469167029</v>
+      </c>
+      <c r="CK22" t="n">
+        <v>2146529.296771839</v>
+      </c>
+      <c r="CL22" t="n">
+        <v>1</v>
+      </c>
+      <c r="CM22" t="n">
+        <v>0.3677411846852089</v>
+      </c>
+      <c r="CN22" t="n">
+        <v>1</v>
+      </c>
+      <c r="CO22" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP22" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ22" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR22" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS22" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT22" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU22" t="n">
+        <v>1</v>
+      </c>
+      <c r="CV22" t="n">
+        <v>3437200000000</v>
+      </c>
+      <c r="CW22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -6716,6 +7804,54 @@
       <c r="CG23" t="n">
         <v>0.03307276007215875</v>
       </c>
+      <c r="CH23" t="n">
+        <v>0.4956607634618106</v>
+      </c>
+      <c r="CI23" t="n">
+        <v>0.289449980846318</v>
+      </c>
+      <c r="CJ23" t="n">
+        <v>0.2592601006024074</v>
+      </c>
+      <c r="CK23" t="n">
+        <v>2422824.025191455</v>
+      </c>
+      <c r="CL23" t="n">
+        <v>0.0289578659920482</v>
+      </c>
+      <c r="CM23" t="n">
+        <v>0.01115909422808121</v>
+      </c>
+      <c r="CN23" t="n">
+        <v>4</v>
+      </c>
+      <c r="CO23" t="n">
+        <v>175.2186374588073</v>
+      </c>
+      <c r="CP23" t="n">
+        <v>45.17356592606907</v>
+      </c>
+      <c r="CQ23" t="n">
+        <v>0.7049143715474392</v>
+      </c>
+      <c r="CR23" t="n">
+        <v>0.2999597455531221</v>
+      </c>
+      <c r="CS23" t="n">
+        <v>1</v>
+      </c>
+      <c r="CT23" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU23" t="n">
+        <v>0</v>
+      </c>
+      <c r="CV23" t="n">
+        <v>0.01010171589423133</v>
+      </c>
+      <c r="CW23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -6983,6 +8119,54 @@
       <c r="CG24" t="n">
         <v>0.0531914893617021</v>
       </c>
+      <c r="CH24" t="n">
+        <v>0.01985610257861567</v>
+      </c>
+      <c r="CI24" t="n">
+        <v>0.2135510350594053</v>
+      </c>
+      <c r="CJ24" t="n">
+        <v>0.1897528629798956</v>
+      </c>
+      <c r="CK24" t="n">
+        <v>1978739.73991409</v>
+      </c>
+      <c r="CL24" t="n">
+        <v>0.224646420348646</v>
+      </c>
+      <c r="CM24" t="n">
+        <v>0.7410371669773052</v>
+      </c>
+      <c r="CN24" t="n">
+        <v>3</v>
+      </c>
+      <c r="CO24" t="n">
+        <v>8.837318225490543</v>
+      </c>
+      <c r="CP24" t="n">
+        <v>6.864095059801242</v>
+      </c>
+      <c r="CQ24" t="n">
+        <v>0.1194057669115229</v>
+      </c>
+      <c r="CR24" t="n">
+        <v>0.1830425349280331</v>
+      </c>
+      <c r="CS24" t="n">
+        <v>0.3527086813236422</v>
+      </c>
+      <c r="CT24" t="n">
+        <v>0.4486807313480212</v>
+      </c>
+      <c r="CU24" t="n">
+        <v>0.5935204473193729</v>
+      </c>
+      <c r="CV24" t="n">
+        <v>3648400000000</v>
+      </c>
+      <c r="CW24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -7250,6 +8434,54 @@
       <c r="CG25" t="n">
         <v>0.1903642773207992</v>
       </c>
+      <c r="CH25" t="n">
+        <v>0.03195132305079949</v>
+      </c>
+      <c r="CI25" t="n">
+        <v>0.2462469335072436</v>
+      </c>
+      <c r="CJ25" t="n">
+        <v>0.258599644582675</v>
+      </c>
+      <c r="CK25" t="n">
+        <v>2058673.312118756</v>
+      </c>
+      <c r="CL25" t="n">
+        <v>-0.07464059412686516</v>
+      </c>
+      <c r="CM25" t="n">
+        <v>0.3649928459494447</v>
+      </c>
+      <c r="CN25" t="n">
+        <v>3</v>
+      </c>
+      <c r="CO25" t="n">
+        <v>173.0787957312185</v>
+      </c>
+      <c r="CP25" t="n">
+        <v>69.97318600476395</v>
+      </c>
+      <c r="CQ25" t="n">
+        <v>0.3749744498194454</v>
+      </c>
+      <c r="CR25" t="n">
+        <v>0.4841163205284962</v>
+      </c>
+      <c r="CS25" t="n">
+        <v>0.1499897799277781</v>
+      </c>
+      <c r="CT25" t="n">
+        <v>0.1936465282113984</v>
+      </c>
+      <c r="CU25" t="n">
+        <v>0.6250255501805546</v>
+      </c>
+      <c r="CV25" t="n">
+        <v>5870800000000</v>
+      </c>
+      <c r="CW25" t="n">
+        <v>0.4</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -7517,6 +8749,54 @@
       <c r="CG26" t="n">
         <v>0.03348214285714284</v>
       </c>
+      <c r="CH26" t="n">
+        <v>0.0356265851030249</v>
+      </c>
+      <c r="CI26" t="n">
+        <v>0.1215051571657122</v>
+      </c>
+      <c r="CJ26" t="n">
+        <v>0.2528568111236079</v>
+      </c>
+      <c r="CK26" t="n">
+        <v>1411029.753981701</v>
+      </c>
+      <c r="CL26" t="n">
+        <v>0.1263500404821191</v>
+      </c>
+      <c r="CM26" t="n">
+        <v>0.382655321489131</v>
+      </c>
+      <c r="CN26" t="n">
+        <v>5</v>
+      </c>
+      <c r="CO26" t="n">
+        <v>179.7470735758901</v>
+      </c>
+      <c r="CP26" t="n">
+        <v>29.49134397786646</v>
+      </c>
+      <c r="CQ26" t="n">
+        <v>0.1195368234521318</v>
+      </c>
+      <c r="CR26" t="n">
+        <v>0.3244191290462165</v>
+      </c>
+      <c r="CS26" t="n">
+        <v>0.1153572356059333</v>
+      </c>
+      <c r="CT26" t="n">
+        <v>0.3168250442449446</v>
+      </c>
+      <c r="CU26" t="n">
+        <v>0.8804631765478682</v>
+      </c>
+      <c r="CV26" t="n">
+        <v>9.346293662068364</v>
+      </c>
+      <c r="CW26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -7784,6 +9064,54 @@
       <c r="CG27" t="n">
         <v>0.3228459063282088</v>
       </c>
+      <c r="CH27" t="n">
+        <v>0.02746350861534108</v>
+      </c>
+      <c r="CI27" t="n">
+        <v>0.2080413603313179</v>
+      </c>
+      <c r="CJ27" t="n">
+        <v>0.2843873048946727</v>
+      </c>
+      <c r="CK27" t="n">
+        <v>1869011.801404102</v>
+      </c>
+      <c r="CL27" t="n">
+        <v>0.2529428084499227</v>
+      </c>
+      <c r="CM27" t="n">
+        <v>0.03860330545757203</v>
+      </c>
+      <c r="CN27" t="n">
+        <v>3</v>
+      </c>
+      <c r="CO27" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP27" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ27" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR27" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS27" t="n">
+        <v>0.1170278392360471</v>
+      </c>
+      <c r="CT27" t="n">
+        <v>0.09200534332279607</v>
+      </c>
+      <c r="CU27" t="n">
+        <v>0.1418889461376878</v>
+      </c>
+      <c r="CV27" t="n">
+        <v>5046200000000</v>
+      </c>
+      <c r="CW27" t="n">
+        <v>0.1254901960784314</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -8051,6 +9379,54 @@
       <c r="CG28" t="n">
         <v>0.1040871934604905</v>
       </c>
+      <c r="CH28" t="n">
+        <v>0.02468515636054903</v>
+      </c>
+      <c r="CI28" t="n">
+        <v>0.146332081173919</v>
+      </c>
+      <c r="CJ28" t="n">
+        <v>0.2133615086068617</v>
+      </c>
+      <c r="CK28" t="n">
+        <v>2219277.180067528</v>
+      </c>
+      <c r="CL28" t="n">
+        <v>0.8143175254095288</v>
+      </c>
+      <c r="CM28" t="n">
+        <v>0.09398769759904756</v>
+      </c>
+      <c r="CN28" t="n">
+        <v>1</v>
+      </c>
+      <c r="CO28" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP28" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ28" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR28" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS28" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT28" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU28" t="n">
+        <v>1</v>
+      </c>
+      <c r="CV28" t="n">
+        <v>4535700000000</v>
+      </c>
+      <c r="CW28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -8318,6 +9694,54 @@
       <c r="CG29" t="n">
         <v>0.3245125348189415</v>
       </c>
+      <c r="CH29" t="n">
+        <v>0.2947741942506341</v>
+      </c>
+      <c r="CI29" t="n">
+        <v>0.2173980878859035</v>
+      </c>
+      <c r="CJ29" t="n">
+        <v>0.2678914941044723</v>
+      </c>
+      <c r="CK29" t="n">
+        <v>1948179.481436119</v>
+      </c>
+      <c r="CL29" t="n">
+        <v>0.3375330487570714</v>
+      </c>
+      <c r="CM29" t="n">
+        <v>0.4371778207760365</v>
+      </c>
+      <c r="CN29" t="n">
+        <v>5</v>
+      </c>
+      <c r="CO29" t="n">
+        <v>127.084594556315</v>
+      </c>
+      <c r="CP29" t="n">
+        <v>28.00474515045933</v>
+      </c>
+      <c r="CQ29" t="n">
+        <v>0.9625496654505709</v>
+      </c>
+      <c r="CR29" t="n">
+        <v>0.18986260029707</v>
+      </c>
+      <c r="CS29" t="n">
+        <v>0.3929839613791841</v>
+      </c>
+      <c r="CT29" t="n">
+        <v>0.09170635941430104</v>
+      </c>
+      <c r="CU29" t="n">
+        <v>0.03232316145517924</v>
+      </c>
+      <c r="CV29" t="n">
+        <v>0.3861032416897532</v>
+      </c>
+      <c r="CW29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -8585,6 +10009,54 @@
       <c r="CG30" t="n">
         <v>0.1606313834726091</v>
       </c>
+      <c r="CH30" t="n">
+        <v>0.02214137214137214</v>
+      </c>
+      <c r="CI30" t="n">
+        <v>0.0855270665276775</v>
+      </c>
+      <c r="CJ30" t="n">
+        <v>0.1034674504847561</v>
+      </c>
+      <c r="CK30" t="n">
+        <v>935241.7642505784</v>
+      </c>
+      <c r="CL30" t="n">
+        <v>0.2104810363050906</v>
+      </c>
+      <c r="CM30" t="n">
+        <v>0.8640218272988718</v>
+      </c>
+      <c r="CN30" t="n">
+        <v>7</v>
+      </c>
+      <c r="CO30" t="n">
+        <v>178.6681454554751</v>
+      </c>
+      <c r="CP30" t="n">
+        <v>37.15757201577725</v>
+      </c>
+      <c r="CQ30" t="n">
+        <v>0.2042523904333506</v>
+      </c>
+      <c r="CR30" t="n">
+        <v>0.3804253611554385</v>
+      </c>
+      <c r="CS30" t="n">
+        <v>0.3311876184733904</v>
+      </c>
+      <c r="CT30" t="n">
+        <v>0.4210294932667076</v>
+      </c>
+      <c r="CU30" t="n">
+        <v>0.5221591328073151</v>
+      </c>
+      <c r="CV30" t="n">
+        <v>4.728386370029952</v>
+      </c>
+      <c r="CW30" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -8852,6 +10324,54 @@
       <c r="CG31" t="n">
         <v>0.1428571428571429</v>
       </c>
+      <c r="CH31" t="n">
+        <v>0.02956809003929423</v>
+      </c>
+      <c r="CI31" t="n">
+        <v>0.1577101372250689</v>
+      </c>
+      <c r="CJ31" t="n">
+        <v>0.1760406976824831</v>
+      </c>
+      <c r="CK31" t="n">
+        <v>1446306.157699465</v>
+      </c>
+      <c r="CL31" t="n">
+        <v>-0.3325479946253382</v>
+      </c>
+      <c r="CM31" t="n">
+        <v>0.4663255351653813</v>
+      </c>
+      <c r="CN31" t="n">
+        <v>5</v>
+      </c>
+      <c r="CO31" t="n">
+        <v>12.48974247801543</v>
+      </c>
+      <c r="CP31" t="n">
+        <v>7.398932912185946</v>
+      </c>
+      <c r="CQ31" t="n">
+        <v>0.2331535643947063</v>
+      </c>
+      <c r="CR31" t="n">
+        <v>0.3163425217420026</v>
+      </c>
+      <c r="CS31" t="n">
+        <v>0.3862894153593628</v>
+      </c>
+      <c r="CT31" t="n">
+        <v>0.4584971995916545</v>
+      </c>
+      <c r="CU31" t="n">
+        <v>0.5492278525281158</v>
+      </c>
+      <c r="CV31" t="n">
+        <v>5432900000000</v>
+      </c>
+      <c r="CW31" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -9119,6 +10639,54 @@
       <c r="CG32" t="n">
         <v>0.2793427230046948</v>
       </c>
+      <c r="CH32" t="n">
+        <v>0.01501289852075192</v>
+      </c>
+      <c r="CI32" t="n">
+        <v>0.121863018503303</v>
+      </c>
+      <c r="CJ32" t="n">
+        <v>0.1685329335612348</v>
+      </c>
+      <c r="CK32" t="n">
+        <v>1400806.777658437</v>
+      </c>
+      <c r="CL32" t="n">
+        <v>-0.648142106217147</v>
+      </c>
+      <c r="CM32" t="n">
+        <v>0.4066340402392605</v>
+      </c>
+      <c r="CN32" t="n">
+        <v>2</v>
+      </c>
+      <c r="CO32" t="n">
+        <v>133.8330581837518</v>
+      </c>
+      <c r="CP32" t="n">
+        <v>51.92569760857439</v>
+      </c>
+      <c r="CQ32" t="n">
+        <v>0.4262461482689868</v>
+      </c>
+      <c r="CR32" t="n">
+        <v>0.4945304534149942</v>
+      </c>
+      <c r="CS32" t="n">
+        <v>0.4262461482689868</v>
+      </c>
+      <c r="CT32" t="n">
+        <v>0.4945304534149942</v>
+      </c>
+      <c r="CU32" t="n">
+        <v>0.5737538517310132</v>
+      </c>
+      <c r="CV32" t="n">
+        <v>1.346062255484482</v>
+      </c>
+      <c r="CW32" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -9386,6 +10954,54 @@
       <c r="CG33" t="n">
         <v>0.3584905660377359</v>
       </c>
+      <c r="CH33" t="n">
+        <v>0.01962915392234764</v>
+      </c>
+      <c r="CI33" t="n">
+        <v>0.2481963469524909</v>
+      </c>
+      <c r="CJ33" t="n">
+        <v>0.2126651782842212</v>
+      </c>
+      <c r="CK33" t="n">
+        <v>2208831.302861665</v>
+      </c>
+      <c r="CL33" t="n">
+        <v>0.1829650372917071</v>
+      </c>
+      <c r="CM33" t="n">
+        <v>-0.5075831092134084</v>
+      </c>
+      <c r="CN33" t="n">
+        <v>1</v>
+      </c>
+      <c r="CO33" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP33" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ33" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR33" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS33" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT33" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU33" t="n">
+        <v>1</v>
+      </c>
+      <c r="CV33" t="n">
+        <v>3606700000000</v>
+      </c>
+      <c r="CW33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -9653,6 +11269,54 @@
       <c r="CG34" t="n">
         <v>0.179936305732484</v>
       </c>
+      <c r="CH34" t="n">
+        <v>0.03797172121779452</v>
+      </c>
+      <c r="CI34" t="n">
+        <v>0.212534671313659</v>
+      </c>
+      <c r="CJ34" t="n">
+        <v>0.2346220985225826</v>
+      </c>
+      <c r="CK34" t="n">
+        <v>1945750.675784997</v>
+      </c>
+      <c r="CL34" t="n">
+        <v>0.1821126558692848</v>
+      </c>
+      <c r="CM34" t="n">
+        <v>-0.2713200515981081</v>
+      </c>
+      <c r="CN34" t="n">
+        <v>4</v>
+      </c>
+      <c r="CO34" t="n">
+        <v>20.69552849845148</v>
+      </c>
+      <c r="CP34" t="n">
+        <v>16.39299352506374</v>
+      </c>
+      <c r="CQ34" t="n">
+        <v>0.3672638669915436</v>
+      </c>
+      <c r="CR34" t="n">
+        <v>0.4820592484269557</v>
+      </c>
+      <c r="CS34" t="n">
+        <v>0.1469055467966174</v>
+      </c>
+      <c r="CT34" t="n">
+        <v>0.1928236993707823</v>
+      </c>
+      <c r="CU34" t="n">
+        <v>0.6327361330084563</v>
+      </c>
+      <c r="CV34" t="n">
+        <v>2.647341732446731</v>
+      </c>
+      <c r="CW34" t="n">
+        <v>0.4</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -9920,6 +11584,54 @@
       <c r="CG35" t="n">
         <v>0.07918968692449367</v>
       </c>
+      <c r="CH35" t="n">
+        <v>0.0298837500408181</v>
+      </c>
+      <c r="CI35" t="n">
+        <v>0.1915729684705899</v>
+      </c>
+      <c r="CJ35" t="n">
+        <v>0.2051983580354106</v>
+      </c>
+      <c r="CK35" t="n">
+        <v>1953666.555886148</v>
+      </c>
+      <c r="CL35" t="n">
+        <v>0.5030687136899233</v>
+      </c>
+      <c r="CM35" t="n">
+        <v>0.0129486969349287</v>
+      </c>
+      <c r="CN35" t="n">
+        <v>1</v>
+      </c>
+      <c r="CO35" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP35" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ35" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR35" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS35" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT35" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU35" t="n">
+        <v>1</v>
+      </c>
+      <c r="CV35" t="n">
+        <v>5490900000000</v>
+      </c>
+      <c r="CW35" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -10187,6 +11899,54 @@
       <c r="CG36" t="n">
         <v>0.3867093674939952</v>
       </c>
+      <c r="CH36" t="n">
+        <v>0.07127548410270923</v>
+      </c>
+      <c r="CI36" t="n">
+        <v>0.2849293326658741</v>
+      </c>
+      <c r="CJ36" t="n">
+        <v>0.1772168558334102</v>
+      </c>
+      <c r="CK36" t="n">
+        <v>2588597.335351799</v>
+      </c>
+      <c r="CL36" t="n">
+        <v>-0.3959515282942511</v>
+      </c>
+      <c r="CM36" t="n">
+        <v>0.4048548063193421</v>
+      </c>
+      <c r="CN36" t="n">
+        <v>3</v>
+      </c>
+      <c r="CO36" t="n">
+        <v>6.911571837259563</v>
+      </c>
+      <c r="CP36" t="n">
+        <v>10.11595638330937</v>
+      </c>
+      <c r="CQ36" t="n">
+        <v>0.2691218130311614</v>
+      </c>
+      <c r="CR36" t="n">
+        <v>0.4435033965844929</v>
+      </c>
+      <c r="CS36" t="n">
+        <v>0.2691218130311614</v>
+      </c>
+      <c r="CT36" t="n">
+        <v>0.4435033965844929</v>
+      </c>
+      <c r="CU36" t="n">
+        <v>0.7308781869688386</v>
+      </c>
+      <c r="CV36" t="n">
+        <v>6.644349754840857</v>
+      </c>
+      <c r="CW36" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -10454,6 +12214,54 @@
       <c r="CG37" t="n">
         <v>0.3076923076923077</v>
       </c>
+      <c r="CH37" t="n">
+        <v>0.01501670821042549</v>
+      </c>
+      <c r="CI37" t="n">
+        <v>0.1574876485815304</v>
+      </c>
+      <c r="CJ37" t="n">
+        <v>0.25700837035145</v>
+      </c>
+      <c r="CK37" t="n">
+        <v>2049624.809966721</v>
+      </c>
+      <c r="CL37" t="n">
+        <v>-0.4575964047550015</v>
+      </c>
+      <c r="CM37" t="n">
+        <v>0.5099304146129313</v>
+      </c>
+      <c r="CN37" t="n">
+        <v>3</v>
+      </c>
+      <c r="CO37" t="n">
+        <v>4.253423048080416</v>
+      </c>
+      <c r="CP37" t="n">
+        <v>8.246584009081879</v>
+      </c>
+      <c r="CQ37" t="n">
+        <v>0.1462380400115976</v>
+      </c>
+      <c r="CR37" t="n">
+        <v>0.3533446980855435</v>
+      </c>
+      <c r="CS37" t="n">
+        <v>0.1462380400115976</v>
+      </c>
+      <c r="CT37" t="n">
+        <v>0.3533446980855435</v>
+      </c>
+      <c r="CU37" t="n">
+        <v>0.8537619599884024</v>
+      </c>
+      <c r="CV37" t="n">
+        <v>11.14436619713405</v>
+      </c>
+      <c r="CW37" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -10721,6 +12529,54 @@
       <c r="CG38" t="n">
         <v>0.3349565217391304</v>
       </c>
+      <c r="CH38" t="n">
+        <v>0.02475100956776349</v>
+      </c>
+      <c r="CI38" t="n">
+        <v>0.1963481555982375</v>
+      </c>
+      <c r="CJ38" t="n">
+        <v>0.2557775915827681</v>
+      </c>
+      <c r="CK38" t="n">
+        <v>2096584.527438897</v>
+      </c>
+      <c r="CL38" t="n">
+        <v>0.5333567878974449</v>
+      </c>
+      <c r="CM38" t="n">
+        <v>-0.4576718413298738</v>
+      </c>
+      <c r="CN38" t="n">
+        <v>2</v>
+      </c>
+      <c r="CO38" t="n">
+        <v>139.3486222731156</v>
+      </c>
+      <c r="CP38" t="n">
+        <v>58.75401351432459</v>
+      </c>
+      <c r="CQ38" t="n">
+        <v>0.3986323057302432</v>
+      </c>
+      <c r="CR38" t="n">
+        <v>0.4896167792860383</v>
+      </c>
+      <c r="CS38" t="n">
+        <v>0.3986323057302432</v>
+      </c>
+      <c r="CT38" t="n">
+        <v>0.4896167792860383</v>
+      </c>
+      <c r="CU38" t="n">
+        <v>0.6013676942697568</v>
+      </c>
+      <c r="CV38" t="n">
+        <v>1.508577417396708</v>
+      </c>
+      <c r="CW38" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -10988,6 +12844,54 @@
       <c r="CG39" t="n">
         <v>0.1309846431797652</v>
       </c>
+      <c r="CH39" t="n">
+        <v>0.01990834975128169</v>
+      </c>
+      <c r="CI39" t="n">
+        <v>0.07707034535306163</v>
+      </c>
+      <c r="CJ39" t="n">
+        <v>0.1254908097884468</v>
+      </c>
+      <c r="CK39" t="n">
+        <v>827400.2474341397</v>
+      </c>
+      <c r="CL39" t="n">
+        <v>0.1296883542919628</v>
+      </c>
+      <c r="CM39" t="n">
+        <v>0.7030071077091307</v>
+      </c>
+      <c r="CN39" t="n">
+        <v>6</v>
+      </c>
+      <c r="CO39" t="n">
+        <v>9.485233167164962</v>
+      </c>
+      <c r="CP39" t="n">
+        <v>13.92293897405934</v>
+      </c>
+      <c r="CQ39" t="n">
+        <v>0.6710934937124111</v>
+      </c>
+      <c r="CR39" t="n">
+        <v>0.4599437250222052</v>
+      </c>
+      <c r="CS39" t="n">
+        <v>0.3996336796063422</v>
+      </c>
+      <c r="CT39" t="n">
+        <v>0.3495195128547631</v>
+      </c>
+      <c r="CU39" t="n">
+        <v>0.3059595407326408</v>
+      </c>
+      <c r="CV39" t="n">
+        <v>5.396223115919923</v>
+      </c>
+      <c r="CW39" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -11255,6 +13159,54 @@
       <c r="CG40" t="n">
         <v>0.2015325670498085</v>
       </c>
+      <c r="CH40" t="n">
+        <v>0.01692808394379075</v>
+      </c>
+      <c r="CI40" t="n">
+        <v>0.2196730783272338</v>
+      </c>
+      <c r="CJ40" t="n">
+        <v>0.1282839797771162</v>
+      </c>
+      <c r="CK40" t="n">
+        <v>2019711.965980136</v>
+      </c>
+      <c r="CL40" t="n">
+        <v>0.003472222222222222</v>
+      </c>
+      <c r="CM40" t="n">
+        <v>0.9315200617283951</v>
+      </c>
+      <c r="CN40" t="n">
+        <v>2</v>
+      </c>
+      <c r="CO40" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP40" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ40" t="n">
+        <v>0.02928883744855967</v>
+      </c>
+      <c r="CR40" t="n">
+        <v>0.168614950254927</v>
+      </c>
+      <c r="CS40" t="n">
+        <v>0.01171553497942387</v>
+      </c>
+      <c r="CT40" t="n">
+        <v>0.06744598010197082</v>
+      </c>
+      <c r="CU40" t="n">
+        <v>0.9707111625514403</v>
+      </c>
+      <c r="CV40" t="n">
+        <v>3110400000000</v>
+      </c>
+      <c r="CW40" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -11522,6 +13474,54 @@
       <c r="CG41" t="n">
         <v>0.3502287926786343</v>
       </c>
+      <c r="CH41" t="n">
+        <v>0.04457826735313646</v>
+      </c>
+      <c r="CI41" t="n">
+        <v>0.2088035552992977</v>
+      </c>
+      <c r="CJ41" t="n">
+        <v>0.2611383565429584</v>
+      </c>
+      <c r="CK41" t="n">
+        <v>1858368.456859014</v>
+      </c>
+      <c r="CL41" t="n">
+        <v>0.1517171495195888</v>
+      </c>
+      <c r="CM41" t="n">
+        <v>-0.2592999548279188</v>
+      </c>
+      <c r="CN41" t="n">
+        <v>6</v>
+      </c>
+      <c r="CO41" t="n">
+        <v>10.04700628458174</v>
+      </c>
+      <c r="CP41" t="n">
+        <v>14.32634659244952</v>
+      </c>
+      <c r="CQ41" t="n">
+        <v>0.1853911047626024</v>
+      </c>
+      <c r="CR41" t="n">
+        <v>0.3875650661956196</v>
+      </c>
+      <c r="CS41" t="n">
+        <v>0.1874275110183252</v>
+      </c>
+      <c r="CT41" t="n">
+        <v>0.3902543262179176</v>
+      </c>
+      <c r="CU41" t="n">
+        <v>0.8125724889816748</v>
+      </c>
+      <c r="CV41" t="n">
+        <v>6.262079971623138</v>
+      </c>
+      <c r="CW41" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -11789,6 +13789,54 @@
       <c r="CG42" t="n">
         <v>0.3450580372845585</v>
       </c>
+      <c r="CH42" t="n">
+        <v>0.06325445461571116</v>
+      </c>
+      <c r="CI42" t="n">
+        <v>0.2600030097157845</v>
+      </c>
+      <c r="CJ42" t="n">
+        <v>0.23290234981597</v>
+      </c>
+      <c r="CK42" t="n">
+        <v>2107729.784322333</v>
+      </c>
+      <c r="CL42" t="n">
+        <v>-0.02315336631533663</v>
+      </c>
+      <c r="CM42" t="n">
+        <v>0.3232781243278124</v>
+      </c>
+      <c r="CN42" t="n">
+        <v>5</v>
+      </c>
+      <c r="CO42" t="n">
+        <v>63.0589419894037</v>
+      </c>
+      <c r="CP42" t="n">
+        <v>34.10045255943876</v>
+      </c>
+      <c r="CQ42" t="n">
+        <v>0.5180262422026242</v>
+      </c>
+      <c r="CR42" t="n">
+        <v>0.4905747325850605</v>
+      </c>
+      <c r="CS42" t="n">
+        <v>0.2387506990750699</v>
+      </c>
+      <c r="CT42" t="n">
+        <v>0.2470366352872888</v>
+      </c>
+      <c r="CU42" t="n">
+        <v>0.4594450419445042</v>
+      </c>
+      <c r="CV42" t="n">
+        <v>1.064350544395115</v>
+      </c>
+      <c r="CW42" t="n">
+        <v>0.4</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -12056,6 +14104,54 @@
       <c r="CG43" t="n">
         <v>0.3886756238003839</v>
       </c>
+      <c r="CH43" t="n">
+        <v>0.08639342121017514</v>
+      </c>
+      <c r="CI43" t="n">
+        <v>0.1935534175583837</v>
+      </c>
+      <c r="CJ43" t="n">
+        <v>0.169824337478055</v>
+      </c>
+      <c r="CK43" t="n">
+        <v>1671748.188693749</v>
+      </c>
+      <c r="CL43" t="n">
+        <v>-0.08042660686275127</v>
+      </c>
+      <c r="CM43" t="n">
+        <v>0.1300042207117254</v>
+      </c>
+      <c r="CN43" t="n">
+        <v>3</v>
+      </c>
+      <c r="CO43" t="n">
+        <v>22.83894277817609</v>
+      </c>
+      <c r="CP43" t="n">
+        <v>6.434271931466984</v>
+      </c>
+      <c r="CQ43" t="n">
+        <v>0.3354445291386598</v>
+      </c>
+      <c r="CR43" t="n">
+        <v>0.2031356202421672</v>
+      </c>
+      <c r="CS43" t="n">
+        <v>0.7895880711347415</v>
+      </c>
+      <c r="CT43" t="n">
+        <v>0.4076012132666681</v>
+      </c>
+      <c r="CU43" t="n">
+        <v>0.2104119288652585</v>
+      </c>
+      <c r="CV43" t="n">
+        <v>15874100000000</v>
+      </c>
+      <c r="CW43" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -12323,6 +14419,54 @@
       <c r="CG44" t="n">
         <v>0.3204903677758318</v>
       </c>
+      <c r="CH44" t="n">
+        <v>0.1833908415060247</v>
+      </c>
+      <c r="CI44" t="n">
+        <v>0.2863627611138915</v>
+      </c>
+      <c r="CJ44" t="n">
+        <v>0.2618135813132149</v>
+      </c>
+      <c r="CK44" t="n">
+        <v>2412121.103046085</v>
+      </c>
+      <c r="CL44" t="n">
+        <v>-0.03764771519975309</v>
+      </c>
+      <c r="CM44" t="n">
+        <v>0.2319165731854252</v>
+      </c>
+      <c r="CN44" t="n">
+        <v>16</v>
+      </c>
+      <c r="CO44" t="n">
+        <v>36.03905242715447</v>
+      </c>
+      <c r="CP44" t="n">
+        <v>44.08972726738016</v>
+      </c>
+      <c r="CQ44" t="n">
+        <v>0.5900162034151814</v>
+      </c>
+      <c r="CR44" t="n">
+        <v>0.4360604508765934</v>
+      </c>
+      <c r="CS44" t="n">
+        <v>0.7144086335352622</v>
+      </c>
+      <c r="CT44" t="n">
+        <v>0.2971117446500878</v>
+      </c>
+      <c r="CU44" t="n">
+        <v>0.01933132719621564</v>
+      </c>
+      <c r="CV44" t="n">
+        <v>0.7066149397053029</v>
+      </c>
+      <c r="CW44" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -12590,6 +14734,54 @@
       <c r="CG45" t="n">
         <v>0.5382989963021658</v>
       </c>
+      <c r="CH45" t="n">
+        <v>0.01558326348902265</v>
+      </c>
+      <c r="CI45" t="n">
+        <v>0.07277419793755864</v>
+      </c>
+      <c r="CJ45" t="n">
+        <v>0.168053299391941</v>
+      </c>
+      <c r="CK45" t="n">
+        <v>1801974.624629322</v>
+      </c>
+      <c r="CL45" t="n">
+        <v>-1</v>
+      </c>
+      <c r="CM45" t="n">
+        <v>0.3239269374497957</v>
+      </c>
+      <c r="CN45" t="n">
+        <v>7</v>
+      </c>
+      <c r="CO45" t="n">
+        <v>178.9769388511433</v>
+      </c>
+      <c r="CP45" t="n">
+        <v>36.42417335789938</v>
+      </c>
+      <c r="CQ45" t="n">
+        <v>0.2522264519959487</v>
+      </c>
+      <c r="CR45" t="n">
+        <v>0.4342905351368875</v>
+      </c>
+      <c r="CS45" t="n">
+        <v>0.2887588227761331</v>
+      </c>
+      <c r="CT45" t="n">
+        <v>0.4083454057091956</v>
+      </c>
+      <c r="CU45" t="n">
+        <v>0.6296580868228967</v>
+      </c>
+      <c r="CV45" t="n">
+        <v>4.952806652796356</v>
+      </c>
+      <c r="CW45" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -12857,6 +15049,54 @@
       <c r="CG46" t="n">
         <v>0.4831460674157303</v>
       </c>
+      <c r="CH46" t="n">
+        <v>0.03540126917090268</v>
+      </c>
+      <c r="CI46" t="n">
+        <v>0.2196305442791445</v>
+      </c>
+      <c r="CJ46" t="n">
+        <v>0.2385928171392352</v>
+      </c>
+      <c r="CK46" t="n">
+        <v>1926103.255145039</v>
+      </c>
+      <c r="CL46" t="n">
+        <v>-0.2114932279736191</v>
+      </c>
+      <c r="CM46" t="n">
+        <v>0.4789921133949298</v>
+      </c>
+      <c r="CN46" t="n">
+        <v>7</v>
+      </c>
+      <c r="CO46" t="n">
+        <v>0.9505195696159884</v>
+      </c>
+      <c r="CP46" t="n">
+        <v>31.97665126507634</v>
+      </c>
+      <c r="CQ46" t="n">
+        <v>0.2234999308192538</v>
+      </c>
+      <c r="CR46" t="n">
+        <v>0.4165905804780547</v>
+      </c>
+      <c r="CS46" t="n">
+        <v>0.2068346357098653</v>
+      </c>
+      <c r="CT46" t="n">
+        <v>0.3399294026836496</v>
+      </c>
+      <c r="CU46" t="n">
+        <v>0.685488954140852</v>
+      </c>
+      <c r="CV46" t="n">
+        <v>8.45038500652557</v>
+      </c>
+      <c r="CW46" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -13124,6 +15364,54 @@
       <c r="CG47" t="n">
         <v>0.1885991510006065</v>
       </c>
+      <c r="CH47" t="n">
+        <v>0.03457783196003091</v>
+      </c>
+      <c r="CI47" t="n">
+        <v>0.2686236371135627</v>
+      </c>
+      <c r="CJ47" t="n">
+        <v>0.2486298693546722</v>
+      </c>
+      <c r="CK47" t="n">
+        <v>2229597.412605859</v>
+      </c>
+      <c r="CL47" t="n">
+        <v>-0.2654956401296943</v>
+      </c>
+      <c r="CM47" t="n">
+        <v>-0.06827840211540277</v>
+      </c>
+      <c r="CN47" t="n">
+        <v>1</v>
+      </c>
+      <c r="CO47" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP47" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ47" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR47" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS47" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT47" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU47" t="n">
+        <v>1</v>
+      </c>
+      <c r="CV47" t="n">
+        <v>6353400000000</v>
+      </c>
+      <c r="CW47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -13391,6 +15679,54 @@
       <c r="CG48" t="n">
         <v>0.1832797427652734</v>
       </c>
+      <c r="CH48" t="n">
+        <v>0.03456368168410053</v>
+      </c>
+      <c r="CI48" t="n">
+        <v>0.1404854055666681</v>
+      </c>
+      <c r="CJ48" t="n">
+        <v>0.2157872499611772</v>
+      </c>
+      <c r="CK48" t="n">
+        <v>2434745.071120878</v>
+      </c>
+      <c r="CL48" t="n">
+        <v>-1</v>
+      </c>
+      <c r="CM48" t="n">
+        <v>-0.6520123449014298</v>
+      </c>
+      <c r="CN48" t="n">
+        <v>1</v>
+      </c>
+      <c r="CO48" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP48" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ48" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR48" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS48" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT48" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU48" t="n">
+        <v>1</v>
+      </c>
+      <c r="CV48" t="n">
+        <v>6350800000000</v>
+      </c>
+      <c r="CW48" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -13658,6 +15994,54 @@
       <c r="CG49" t="n">
         <v>0.2993348115299335</v>
       </c>
+      <c r="CH49" t="n">
+        <v>0.0142896017241567</v>
+      </c>
+      <c r="CI49" t="n">
+        <v>0.0836291978666496</v>
+      </c>
+      <c r="CJ49" t="n">
+        <v>0.1417208101904417</v>
+      </c>
+      <c r="CK49" t="n">
+        <v>980293.9944392436</v>
+      </c>
+      <c r="CL49" t="n">
+        <v>-0.4245886654478976</v>
+      </c>
+      <c r="CM49" t="n">
+        <v>0.6384826325411335</v>
+      </c>
+      <c r="CN49" t="n">
+        <v>2</v>
+      </c>
+      <c r="CO49" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP49" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ49" t="n">
+        <v>0.0184338817794028</v>
+      </c>
+      <c r="CR49" t="n">
+        <v>0.1345142140516972</v>
+      </c>
+      <c r="CS49" t="n">
+        <v>0.0184338817794028</v>
+      </c>
+      <c r="CT49" t="n">
+        <v>0.1345142140516972</v>
+      </c>
+      <c r="CU49" t="n">
+        <v>0.9815661182205973</v>
+      </c>
+      <c r="CV49" t="n">
+        <v>2625600000000</v>
+      </c>
+      <c r="CW49" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -13925,6 +16309,54 @@
       <c r="CG50" t="n">
         <v>0.3280276816608996</v>
       </c>
+      <c r="CH50" t="n">
+        <v>0.6933139946228951</v>
+      </c>
+      <c r="CI50" t="n">
+        <v>0.2858600593294714</v>
+      </c>
+      <c r="CJ50" t="n">
+        <v>0.2508497065883861</v>
+      </c>
+      <c r="CK50" t="n">
+        <v>2370560.035988438</v>
+      </c>
+      <c r="CL50" t="n">
+        <v>-0.02577656645804371</v>
+      </c>
+      <c r="CM50" t="n">
+        <v>-0.3849152490484014</v>
+      </c>
+      <c r="CN50" t="n">
+        <v>6</v>
+      </c>
+      <c r="CO50" t="n">
+        <v>33.42930223321311</v>
+      </c>
+      <c r="CP50" t="n">
+        <v>29.93457525179234</v>
+      </c>
+      <c r="CQ50" t="n">
+        <v>0.4999658531339365</v>
+      </c>
+      <c r="CR50" t="n">
+        <v>0.2289317520507258</v>
+      </c>
+      <c r="CS50" t="n">
+        <v>0.9987882964952755</v>
+      </c>
+      <c r="CT50" t="n">
+        <v>0.01552006686717313</v>
+      </c>
+      <c r="CU50" t="n">
+        <v>0</v>
+      </c>
+      <c r="CV50" t="n">
+        <v>3.507992172377428</v>
+      </c>
+      <c r="CW50" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -14192,6 +16624,54 @@
       <c r="CG51" t="n">
         <v>0.4401709401709402</v>
       </c>
+      <c r="CH51" t="n">
+        <v>0.1220450414167692</v>
+      </c>
+      <c r="CI51" t="n">
+        <v>0.2389666346472196</v>
+      </c>
+      <c r="CJ51" t="n">
+        <v>0.2552044887384488</v>
+      </c>
+      <c r="CK51" t="n">
+        <v>2417749.943924569</v>
+      </c>
+      <c r="CL51" t="n">
+        <v>-0.5952962791195462</v>
+      </c>
+      <c r="CM51" t="n">
+        <v>-0.2313688416396133</v>
+      </c>
+      <c r="CN51" t="n">
+        <v>5</v>
+      </c>
+      <c r="CO51" t="n">
+        <v>70.58277448884664</v>
+      </c>
+      <c r="CP51" t="n">
+        <v>37.7377746948593</v>
+      </c>
+      <c r="CQ51" t="n">
+        <v>0.7052950305019443</v>
+      </c>
+      <c r="CR51" t="n">
+        <v>0.4559100245127384</v>
+      </c>
+      <c r="CS51" t="n">
+        <v>0.4967432765264788</v>
+      </c>
+      <c r="CT51" t="n">
+        <v>0.3834077849115277</v>
+      </c>
+      <c r="CU51" t="n">
+        <v>0.2512976704363027</v>
+      </c>
+      <c r="CV51" t="n">
+        <v>0.5349674522392903</v>
+      </c>
+      <c r="CW51" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -14459,6 +16939,54 @@
       <c r="CG52" t="n">
         <v>0.2589473684210528</v>
       </c>
+      <c r="CH52" t="n">
+        <v>0.0348488641682359</v>
+      </c>
+      <c r="CI52" t="n">
+        <v>0.2124318025435676</v>
+      </c>
+      <c r="CJ52" t="n">
+        <v>0.2308374380158446</v>
+      </c>
+      <c r="CK52" t="n">
+        <v>1823883.120752166</v>
+      </c>
+      <c r="CL52" t="n">
+        <v>-0.06752873563218391</v>
+      </c>
+      <c r="CM52" t="n">
+        <v>0.4440279860069965</v>
+      </c>
+      <c r="CN52" t="n">
+        <v>4</v>
+      </c>
+      <c r="CO52" t="n">
+        <v>1.650037192365639</v>
+      </c>
+      <c r="CP52" t="n">
+        <v>9.219688671295163</v>
+      </c>
+      <c r="CQ52" t="n">
+        <v>0.06974637681159421</v>
+      </c>
+      <c r="CR52" t="n">
+        <v>0.2547190996632355</v>
+      </c>
+      <c r="CS52" t="n">
+        <v>0.07349456399251354</v>
+      </c>
+      <c r="CT52" t="n">
+        <v>0.1795509581898563</v>
+      </c>
+      <c r="CU52" t="n">
+        <v>0.8473888055972014</v>
+      </c>
+      <c r="CV52" t="n">
+        <v>148.9578454297668</v>
+      </c>
+      <c r="CW52" t="n">
+        <v>0.5019607843137255</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -14726,6 +17254,54 @@
       <c r="CG53" t="n">
         <v>0.3212627669452183</v>
       </c>
+      <c r="CH53" t="n">
+        <v>0.0235721827344864</v>
+      </c>
+      <c r="CI53" t="n">
+        <v>0.1926030262951449</v>
+      </c>
+      <c r="CJ53" t="n">
+        <v>0.2028542927503904</v>
+      </c>
+      <c r="CK53" t="n">
+        <v>1713424.002901271</v>
+      </c>
+      <c r="CL53" t="n">
+        <v>0.3499261174732176</v>
+      </c>
+      <c r="CM53" t="n">
+        <v>0.1499353527890654</v>
+      </c>
+      <c r="CN53" t="n">
+        <v>1</v>
+      </c>
+      <c r="CO53" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP53" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ53" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR53" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS53" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT53" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU53" t="n">
+        <v>1</v>
+      </c>
+      <c r="CV53" t="n">
+        <v>4331200000000</v>
+      </c>
+      <c r="CW53" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -14993,6 +17569,54 @@
       <c r="CG54" t="n">
         <v>0.1778140293637847</v>
       </c>
+      <c r="CH54" t="n">
+        <v>0.02664986774934419</v>
+      </c>
+      <c r="CI54" t="n">
+        <v>0.1246293754174835</v>
+      </c>
+      <c r="CJ54" t="n">
+        <v>0.2369484168162398</v>
+      </c>
+      <c r="CK54" t="n">
+        <v>1852564.395647644</v>
+      </c>
+      <c r="CL54" t="n">
+        <v>-0.841893520125799</v>
+      </c>
+      <c r="CM54" t="n">
+        <v>0.5554148712398146</v>
+      </c>
+      <c r="CN54" t="n">
+        <v>5</v>
+      </c>
+      <c r="CO54" t="n">
+        <v>11.5276998263493</v>
+      </c>
+      <c r="CP54" t="n">
+        <v>8.52389380264483</v>
+      </c>
+      <c r="CQ54" t="n">
+        <v>0.3599567055363816</v>
+      </c>
+      <c r="CR54" t="n">
+        <v>0.4799873703294455</v>
+      </c>
+      <c r="CS54" t="n">
+        <v>0.1890906120448465</v>
+      </c>
+      <c r="CT54" t="n">
+        <v>0.2758587127248407</v>
+      </c>
+      <c r="CU54" t="n">
+        <v>0.6215206159250107</v>
+      </c>
+      <c r="CV54" t="n">
+        <v>22.74733268660161</v>
+      </c>
+      <c r="CW54" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -15260,6 +17884,54 @@
       <c r="CG55" t="n">
         <v>0.2618825722273998</v>
       </c>
+      <c r="CH55" t="n">
+        <v>0.02892588520860772</v>
+      </c>
+      <c r="CI55" t="n">
+        <v>0.06329477055508018</v>
+      </c>
+      <c r="CJ55" t="n">
+        <v>0.1185277573824326</v>
+      </c>
+      <c r="CK55" t="n">
+        <v>1202619.17044983</v>
+      </c>
+      <c r="CL55" t="n">
+        <v>0.8764228866018176</v>
+      </c>
+      <c r="CM55" t="n">
+        <v>0.7361380270560124</v>
+      </c>
+      <c r="CN55" t="n">
+        <v>4</v>
+      </c>
+      <c r="CO55" t="n">
+        <v>3.306730083431465</v>
+      </c>
+      <c r="CP55" t="n">
+        <v>4.763400703735601</v>
+      </c>
+      <c r="CQ55" t="n">
+        <v>0.6157218386046774</v>
+      </c>
+      <c r="CR55" t="n">
+        <v>0.4864241524327848</v>
+      </c>
+      <c r="CS55" t="n">
+        <v>0.3334913057962465</v>
+      </c>
+      <c r="CT55" t="n">
+        <v>0.1334475751203792</v>
+      </c>
+      <c r="CU55" t="n">
+        <v>0</v>
+      </c>
+      <c r="CV55" t="n">
+        <v>5314900000000</v>
+      </c>
+      <c r="CW55" t="n">
+        <v>0.3764705882352941</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -15527,6 +18199,54 @@
       <c r="CG56" t="n">
         <v>0.1476971942826892</v>
       </c>
+      <c r="CH56" t="n">
+        <v>0.02147249948297069</v>
+      </c>
+      <c r="CI56" t="n">
+        <v>0.0504268825878432</v>
+      </c>
+      <c r="CJ56" t="n">
+        <v>0.1570573138267009</v>
+      </c>
+      <c r="CK56" t="n">
+        <v>865097.8857773842</v>
+      </c>
+      <c r="CL56" t="n">
+        <v>-0.9023673138338318</v>
+      </c>
+      <c r="CM56" t="n">
+        <v>0.2703401429512851</v>
+      </c>
+      <c r="CN56" t="n">
+        <v>3</v>
+      </c>
+      <c r="CO56" t="n">
+        <v>179.8267045787617</v>
+      </c>
+      <c r="CP56" t="n">
+        <v>8.096493683638277</v>
+      </c>
+      <c r="CQ56" t="n">
+        <v>0.005981649515891925</v>
+      </c>
+      <c r="CR56" t="n">
+        <v>0.07710946365369788</v>
+      </c>
+      <c r="CS56" t="n">
+        <v>0.008627967839439725</v>
+      </c>
+      <c r="CT56" t="n">
+        <v>0.0789892061750305</v>
+      </c>
+      <c r="CU56" t="n">
+        <v>0.9729305013433366</v>
+      </c>
+      <c r="CV56" t="n">
+        <v>166.1779660946535</v>
+      </c>
+      <c r="CW56" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -15794,6 +18514,54 @@
       <c r="CG57" t="n">
         <v>0.1154285714285714</v>
       </c>
+      <c r="CH57" t="n">
+        <v>0.005751542924317793</v>
+      </c>
+      <c r="CI57" t="n">
+        <v>0.06314889478756792</v>
+      </c>
+      <c r="CJ57" t="n">
+        <v>0.1114733112682041</v>
+      </c>
+      <c r="CK57" t="n">
+        <v>890897.98411135</v>
+      </c>
+      <c r="CL57" t="n">
+        <v>0.05866767600302801</v>
+      </c>
+      <c r="CM57" t="n">
+        <v>0.9788039364118092</v>
+      </c>
+      <c r="CN57" t="n">
+        <v>1</v>
+      </c>
+      <c r="CO57" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP57" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ57" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR57" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS57" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT57" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU57" t="n">
+        <v>1</v>
+      </c>
+      <c r="CV57" t="n">
+        <v>1056800000000</v>
+      </c>
+      <c r="CW57" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -16061,6 +18829,54 @@
       <c r="CG58" t="n">
         <v>0.3373403456048084</v>
       </c>
+      <c r="CH58" t="n">
+        <v>0.1148409182440596</v>
+      </c>
+      <c r="CI58" t="n">
+        <v>0.1853734505331721</v>
+      </c>
+      <c r="CJ58" t="n">
+        <v>0.1580649185139597</v>
+      </c>
+      <c r="CK58" t="n">
+        <v>1562811.32216688</v>
+      </c>
+      <c r="CL58" t="n">
+        <v>-0.3599764941164205</v>
+      </c>
+      <c r="CM58" t="n">
+        <v>0.0687784049172792</v>
+      </c>
+      <c r="CN58" t="n">
+        <v>12</v>
+      </c>
+      <c r="CO58" t="n">
+        <v>64.57265793739528</v>
+      </c>
+      <c r="CP58" t="n">
+        <v>23.81629897940758</v>
+      </c>
+      <c r="CQ58" t="n">
+        <v>0.8149470880664988</v>
+      </c>
+      <c r="CR58" t="n">
+        <v>0.3793143865484607</v>
+      </c>
+      <c r="CS58" t="n">
+        <v>0.709959363701976</v>
+      </c>
+      <c r="CT58" t="n">
+        <v>0.3400632686451273</v>
+      </c>
+      <c r="CU58" t="n">
+        <v>0.07747463402381867</v>
+      </c>
+      <c r="CV58" t="n">
+        <v>0.5231382230017595</v>
+      </c>
+      <c r="CW58" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -16328,6 +19144,54 @@
       <c r="CG59" t="n">
         <v>0.1994645247657296</v>
       </c>
+      <c r="CH59" t="n">
+        <v>0.04438070773149307</v>
+      </c>
+      <c r="CI59" t="n">
+        <v>0.1296195729030107</v>
+      </c>
+      <c r="CJ59" t="n">
+        <v>0.1695195010521908</v>
+      </c>
+      <c r="CK59" t="n">
+        <v>1466562.90896555</v>
+      </c>
+      <c r="CL59" t="n">
+        <v>0.3873396610502048</v>
+      </c>
+      <c r="CM59" t="n">
+        <v>0.6366713266131999</v>
+      </c>
+      <c r="CN59" t="n">
+        <v>8</v>
+      </c>
+      <c r="CO59" t="n">
+        <v>15.13635707247538</v>
+      </c>
+      <c r="CP59" t="n">
+        <v>20.22526200376658</v>
+      </c>
+      <c r="CQ59" t="n">
+        <v>0.2495646628896574</v>
+      </c>
+      <c r="CR59" t="n">
+        <v>0.4327610679421487</v>
+      </c>
+      <c r="CS59" t="n">
+        <v>0.2466153351194057</v>
+      </c>
+      <c r="CT59" t="n">
+        <v>0.3193241152224401</v>
+      </c>
+      <c r="CU59" t="n">
+        <v>0.5758467613371594</v>
+      </c>
+      <c r="CV59" t="n">
+        <v>3.999448225121697</v>
+      </c>
+      <c r="CW59" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -16595,6 +19459,54 @@
       <c r="CG60" t="n">
         <v>0.3148418491484186</v>
       </c>
+      <c r="CH60" t="n">
+        <v>0.01458784600145857</v>
+      </c>
+      <c r="CI60" t="n">
+        <v>0.06585984488896632</v>
+      </c>
+      <c r="CJ60" t="n">
+        <v>0.1384484034907968</v>
+      </c>
+      <c r="CK60" t="n">
+        <v>1296926.51046278</v>
+      </c>
+      <c r="CL60" t="n">
+        <v>0.9392627965975228</v>
+      </c>
+      <c r="CM60" t="n">
+        <v>0.5771526637815252</v>
+      </c>
+      <c r="CN60" t="n">
+        <v>1</v>
+      </c>
+      <c r="CO60" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP60" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ60" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR60" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS60" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT60" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU60" t="n">
+        <v>1</v>
+      </c>
+      <c r="CV60" t="n">
+        <v>2680400000000</v>
+      </c>
+      <c r="CW60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -16862,6 +19774,54 @@
       <c r="CG61" t="n">
         <v>0.4215838509316771</v>
       </c>
+      <c r="CH61" t="n">
+        <v>0.02245158972907664</v>
+      </c>
+      <c r="CI61" t="n">
+        <v>0.1825696756815269</v>
+      </c>
+      <c r="CJ61" t="n">
+        <v>0.1815712078066321</v>
+      </c>
+      <c r="CK61" t="n">
+        <v>1590270.772735023</v>
+      </c>
+      <c r="CL61" t="n">
+        <v>-0.2027731316510314</v>
+      </c>
+      <c r="CM61" t="n">
+        <v>0.5193076867136935</v>
+      </c>
+      <c r="CN61" t="n">
+        <v>1</v>
+      </c>
+      <c r="CO61" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP61" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ61" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR61" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS61" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT61" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU61" t="n">
+        <v>1</v>
+      </c>
+      <c r="CV61" t="n">
+        <v>4125300000000</v>
+      </c>
+      <c r="CW61" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -17129,6 +20089,54 @@
       <c r="CG62" t="n">
         <v>0.04040404040404041</v>
       </c>
+      <c r="CH62" t="n">
+        <v>0.2412600276474622</v>
+      </c>
+      <c r="CI62" t="n">
+        <v>0.3176452669163226</v>
+      </c>
+      <c r="CJ62" t="n">
+        <v>0.2222515201114482</v>
+      </c>
+      <c r="CK62" t="n">
+        <v>2554202.495678432</v>
+      </c>
+      <c r="CL62" t="n">
+        <v>0.03076048509348156</v>
+      </c>
+      <c r="CM62" t="n">
+        <v>-0.02804897856060059</v>
+      </c>
+      <c r="CN62" t="n">
+        <v>6</v>
+      </c>
+      <c r="CO62" t="n">
+        <v>104.3796425606961</v>
+      </c>
+      <c r="CP62" t="n">
+        <v>25.70516448974857</v>
+      </c>
+      <c r="CQ62" t="n">
+        <v>0.9200015339637624</v>
+      </c>
+      <c r="CR62" t="n">
+        <v>0.2712908245187931</v>
+      </c>
+      <c r="CS62" t="n">
+        <v>0.5434277879924078</v>
+      </c>
+      <c r="CT62" t="n">
+        <v>0.2721749400270086</v>
+      </c>
+      <c r="CU62" t="n">
+        <v>0.008662383599220386</v>
+      </c>
+      <c r="CV62" t="n">
+        <v>0.0869547094031114</v>
+      </c>
+      <c r="CW62" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -17396,6 +20404,54 @@
       <c r="CG63" t="n">
         <v>0.3444444444444444</v>
       </c>
+      <c r="CH63" t="n">
+        <v>0.05511641323159648</v>
+      </c>
+      <c r="CI63" t="n">
+        <v>0.169402100388071</v>
+      </c>
+      <c r="CJ63" t="n">
+        <v>0.1517403388514831</v>
+      </c>
+      <c r="CK63" t="n">
+        <v>1570684.265194673</v>
+      </c>
+      <c r="CL63" t="n">
+        <v>0.4749782763251442</v>
+      </c>
+      <c r="CM63" t="n">
+        <v>0.2590449482581563</v>
+      </c>
+      <c r="CN63" t="n">
+        <v>6</v>
+      </c>
+      <c r="CO63" t="n">
+        <v>2.884447531750515</v>
+      </c>
+      <c r="CP63" t="n">
+        <v>21.59028068681508</v>
+      </c>
+      <c r="CQ63" t="n">
+        <v>0.1792183426810965</v>
+      </c>
+      <c r="CR63" t="n">
+        <v>0.3804112037004793</v>
+      </c>
+      <c r="CS63" t="n">
+        <v>0.1375714635328814</v>
+      </c>
+      <c r="CT63" t="n">
+        <v>0.258068343194049</v>
+      </c>
+      <c r="CU63" t="n">
+        <v>0.7416067619875187</v>
+      </c>
+      <c r="CV63" t="n">
+        <v>27.86887115157392</v>
+      </c>
+      <c r="CW63" t="n">
+        <v>0.5019607843137255</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -17663,6 +20719,54 @@
       <c r="CG64" t="n">
         <v>0.01836884643644368</v>
       </c>
+      <c r="CH64" t="n">
+        <v>0.1386307975313211</v>
+      </c>
+      <c r="CI64" t="n">
+        <v>0.09723023707961186</v>
+      </c>
+      <c r="CJ64" t="n">
+        <v>0.1257344890888339</v>
+      </c>
+      <c r="CK64" t="n">
+        <v>1300483.495415606</v>
+      </c>
+      <c r="CL64" t="n">
+        <v>-0.09544878161767881</v>
+      </c>
+      <c r="CM64" t="n">
+        <v>-0.9565959885836772</v>
+      </c>
+      <c r="CN64" t="n">
+        <v>8</v>
+      </c>
+      <c r="CO64" t="n">
+        <v>83.83550074375387</v>
+      </c>
+      <c r="CP64" t="n">
+        <v>35.29614064265328</v>
+      </c>
+      <c r="CQ64" t="n">
+        <v>0.6716825728340197</v>
+      </c>
+      <c r="CR64" t="n">
+        <v>0.4696009946593933</v>
+      </c>
+      <c r="CS64" t="n">
+        <v>0.4492269765088151</v>
+      </c>
+      <c r="CT64" t="n">
+        <v>0.2294851433189162</v>
+      </c>
+      <c r="CU64" t="n">
+        <v>0.1074814602529022</v>
+      </c>
+      <c r="CV64" t="n">
+        <v>0.9682192585265599</v>
+      </c>
+      <c r="CW64" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -17930,6 +21034,54 @@
       <c r="CG65" t="n">
         <v>0.4532453245324532</v>
       </c>
+      <c r="CH65" t="n">
+        <v>0.01544992435044791</v>
+      </c>
+      <c r="CI65" t="n">
+        <v>0.1765267350447313</v>
+      </c>
+      <c r="CJ65" t="n">
+        <v>0.1424992504356306</v>
+      </c>
+      <c r="CK65" t="n">
+        <v>1787419.120546625</v>
+      </c>
+      <c r="CL65" t="n">
+        <v>-0.7549668874172185</v>
+      </c>
+      <c r="CM65" t="n">
+        <v>0.7632098069606876</v>
+      </c>
+      <c r="CN65" t="n">
+        <v>2</v>
+      </c>
+      <c r="CO65" t="n">
+        <v>5.391846448876762</v>
+      </c>
+      <c r="CP65" t="n">
+        <v>9.132602028471258</v>
+      </c>
+      <c r="CQ65" t="n">
+        <v>0.1033535296604199</v>
+      </c>
+      <c r="CR65" t="n">
+        <v>0.3044200676157086</v>
+      </c>
+      <c r="CS65" t="n">
+        <v>0.1033535296604199</v>
+      </c>
+      <c r="CT65" t="n">
+        <v>0.3044200676157086</v>
+      </c>
+      <c r="CU65" t="n">
+        <v>0.8966464703395801</v>
+      </c>
+      <c r="CV65" t="n">
+        <v>8.675528288995652</v>
+      </c>
+      <c r="CW65" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -18197,6 +21349,54 @@
       <c r="CG66" t="n">
         <v>0.3284873658705434</v>
       </c>
+      <c r="CH66" t="n">
+        <v>0.02280208117904453</v>
+      </c>
+      <c r="CI66" t="n">
+        <v>0.2957373457094888</v>
+      </c>
+      <c r="CJ66" t="n">
+        <v>0.2480525990932649</v>
+      </c>
+      <c r="CK66" t="n">
+        <v>2596829.706228014</v>
+      </c>
+      <c r="CL66" t="n">
+        <v>0.03477575960092608</v>
+      </c>
+      <c r="CM66" t="n">
+        <v>-0.2884454734229181</v>
+      </c>
+      <c r="CN66" t="n">
+        <v>4</v>
+      </c>
+      <c r="CO66" t="n">
+        <v>179.9895869371301</v>
+      </c>
+      <c r="CP66" t="n">
+        <v>7.100272814109625</v>
+      </c>
+      <c r="CQ66" t="n">
+        <v>0.006802396352960833</v>
+      </c>
+      <c r="CR66" t="n">
+        <v>0.08219564317418566</v>
+      </c>
+      <c r="CS66" t="n">
+        <v>0.006802396352960833</v>
+      </c>
+      <c r="CT66" t="n">
+        <v>0.08219564317418566</v>
+      </c>
+      <c r="CU66" t="n">
+        <v>0.9931976036470391</v>
+      </c>
+      <c r="CV66" t="n">
+        <v>179.5905172336383</v>
+      </c>
+      <c r="CW66" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -18464,6 +21664,54 @@
       <c r="CG67" t="n">
         <v>0.4286778398510243</v>
       </c>
+      <c r="CH67" t="n">
+        <v>0.2581423953151702</v>
+      </c>
+      <c r="CI67" t="n">
+        <v>0.3469651687781321</v>
+      </c>
+      <c r="CJ67" t="n">
+        <v>0.1936675853533001</v>
+      </c>
+      <c r="CK67" t="n">
+        <v>3052772.157758437</v>
+      </c>
+      <c r="CL67" t="n">
+        <v>-0.07966840671619764</v>
+      </c>
+      <c r="CM67" t="n">
+        <v>-0.7446301621703675</v>
+      </c>
+      <c r="CN67" t="n">
+        <v>8</v>
+      </c>
+      <c r="CO67" t="n">
+        <v>50.27926172408046</v>
+      </c>
+      <c r="CP67" t="n">
+        <v>17.35488966018104</v>
+      </c>
+      <c r="CQ67" t="n">
+        <v>0.481692795520286</v>
+      </c>
+      <c r="CR67" t="n">
+        <v>0.2980152570326879</v>
+      </c>
+      <c r="CS67" t="n">
+        <v>0.8628347131530911</v>
+      </c>
+      <c r="CT67" t="n">
+        <v>0.3103545696041367</v>
+      </c>
+      <c r="CU67" t="n">
+        <v>0.04264456606987747</v>
+      </c>
+      <c r="CV67" t="n">
+        <v>1.165678149898355</v>
+      </c>
+      <c r="CW67" t="n">
+        <v>0.8745098039215686</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -18731,6 +21979,54 @@
       <c r="CG68" t="n">
         <v>0.1701081612586037</v>
       </c>
+      <c r="CH68" t="n">
+        <v>0.1219612282439508</v>
+      </c>
+      <c r="CI68" t="n">
+        <v>0.1162144131115993</v>
+      </c>
+      <c r="CJ68" t="n">
+        <v>0.1401703277876162</v>
+      </c>
+      <c r="CK68" t="n">
+        <v>1006645.417407144</v>
+      </c>
+      <c r="CL68" t="n">
+        <v>-0.01634135675207725</v>
+      </c>
+      <c r="CM68" t="n">
+        <v>-0.1467062928949459</v>
+      </c>
+      <c r="CN68" t="n">
+        <v>7</v>
+      </c>
+      <c r="CO68" t="n">
+        <v>26.68676779794189</v>
+      </c>
+      <c r="CP68" t="n">
+        <v>12.39508613205337</v>
+      </c>
+      <c r="CQ68" t="n">
+        <v>0.8245450569850152</v>
+      </c>
+      <c r="CR68" t="n">
+        <v>0.375254649607548</v>
+      </c>
+      <c r="CS68" t="n">
+        <v>0.3803055860487117</v>
+      </c>
+      <c r="CT68" t="n">
+        <v>0.2326435147598716</v>
+      </c>
+      <c r="CU68" t="n">
+        <v>0.1658188081787107</v>
+      </c>
+      <c r="CV68" t="n">
+        <v>20.79478700639876</v>
+      </c>
+      <c r="CW68" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -18998,6 +22294,54 @@
       <c r="CG69" t="n">
         <v>0.3277950848044306</v>
       </c>
+      <c r="CH69" t="n">
+        <v>0.09244919506699611</v>
+      </c>
+      <c r="CI69" t="n">
+        <v>0.1978194168007092</v>
+      </c>
+      <c r="CJ69" t="n">
+        <v>0.1999570356725683</v>
+      </c>
+      <c r="CK69" t="n">
+        <v>1654210.1615847</v>
+      </c>
+      <c r="CL69" t="n">
+        <v>-0.01981538606447359</v>
+      </c>
+      <c r="CM69" t="n">
+        <v>0.2320272211364118</v>
+      </c>
+      <c r="CN69" t="n">
+        <v>12</v>
+      </c>
+      <c r="CO69" t="n">
+        <v>178.2181008717295</v>
+      </c>
+      <c r="CP69" t="n">
+        <v>38.90783970091887</v>
+      </c>
+      <c r="CQ69" t="n">
+        <v>0.6286410624720371</v>
+      </c>
+      <c r="CR69" t="n">
+        <v>0.4678060351639201</v>
+      </c>
+      <c r="CS69" t="n">
+        <v>0.5571187454895773</v>
+      </c>
+      <c r="CT69" t="n">
+        <v>0.3541605737617346</v>
+      </c>
+      <c r="CU69" t="n">
+        <v>0.1621435467539501</v>
+      </c>
+      <c r="CV69" t="n">
+        <v>4.059962467604761</v>
+      </c>
+      <c r="CW69" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -19265,6 +22609,54 @@
       <c r="CG70" t="n">
         <v>0.3507549361207897</v>
       </c>
+      <c r="CH70" t="n">
+        <v>0.08280632626182365</v>
+      </c>
+      <c r="CI70" t="n">
+        <v>0.1310750303679397</v>
+      </c>
+      <c r="CJ70" t="n">
+        <v>0.1307421176857722</v>
+      </c>
+      <c r="CK70" t="n">
+        <v>1422915.27225473</v>
+      </c>
+      <c r="CL70" t="n">
+        <v>-0.6317712783437397</v>
+      </c>
+      <c r="CM70" t="n">
+        <v>0.6661715412421952</v>
+      </c>
+      <c r="CN70" t="n">
+        <v>3</v>
+      </c>
+      <c r="CO70" t="n">
+        <v>149.0963865423799</v>
+      </c>
+      <c r="CP70" t="n">
+        <v>56.81862017927981</v>
+      </c>
+      <c r="CQ70" t="n">
+        <v>0.3393493263227079</v>
+      </c>
+      <c r="CR70" t="n">
+        <v>0.4734885014939985</v>
+      </c>
+      <c r="CS70" t="n">
+        <v>0.3070134348843053</v>
+      </c>
+      <c r="CT70" t="n">
+        <v>0.2145025081033743</v>
+      </c>
+      <c r="CU70" t="n">
+        <v>0.3194413407821229</v>
+      </c>
+      <c r="CV70" t="n">
+        <v>1.946815928106224</v>
+      </c>
+      <c r="CW70" t="n">
+        <v>0.5019607843137255</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -19532,6 +22924,54 @@
       <c r="CG71" t="n">
         <v>0.2905826310003664</v>
       </c>
+      <c r="CH71" t="n">
+        <v>0.03785362083791403</v>
+      </c>
+      <c r="CI71" t="n">
+        <v>0.1439059459573889</v>
+      </c>
+      <c r="CJ71" t="n">
+        <v>0.180551420226541</v>
+      </c>
+      <c r="CK71" t="n">
+        <v>1157358.088429196</v>
+      </c>
+      <c r="CL71" t="n">
+        <v>-0.2889163659367677</v>
+      </c>
+      <c r="CM71" t="n">
+        <v>-0.06031371759665291</v>
+      </c>
+      <c r="CN71" t="n">
+        <v>5</v>
+      </c>
+      <c r="CO71" t="n">
+        <v>7.153797855045158</v>
+      </c>
+      <c r="CP71" t="n">
+        <v>10.56846419837576</v>
+      </c>
+      <c r="CQ71" t="n">
+        <v>0.5093669575719235</v>
+      </c>
+      <c r="CR71" t="n">
+        <v>0.4999122524062055</v>
+      </c>
+      <c r="CS71" t="n">
+        <v>0.216400696548802</v>
+      </c>
+      <c r="CT71" t="n">
+        <v>0.2114811141047654</v>
+      </c>
+      <c r="CU71" t="n">
+        <v>0.4736388078156226</v>
+      </c>
+      <c r="CV71" t="n">
+        <v>144.5083681978136</v>
+      </c>
+      <c r="CW71" t="n">
+        <v>0.4</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -19799,6 +23239,54 @@
       <c r="CG72" t="n">
         <v>0.3929430633520449</v>
       </c>
+      <c r="CH72" t="n">
+        <v>0.02571377257241132</v>
+      </c>
+      <c r="CI72" t="n">
+        <v>0.1346743333517721</v>
+      </c>
+      <c r="CJ72" t="n">
+        <v>0.1890929235177886</v>
+      </c>
+      <c r="CK72" t="n">
+        <v>2167966.424535499</v>
+      </c>
+      <c r="CL72" t="n">
+        <v>0.8443075750841323</v>
+      </c>
+      <c r="CM72" t="n">
+        <v>0.2283954536795987</v>
+      </c>
+      <c r="CN72" t="n">
+        <v>2</v>
+      </c>
+      <c r="CO72" t="n">
+        <v>1.310730703773072</v>
+      </c>
+      <c r="CP72" t="n">
+        <v>4.780816603682069</v>
+      </c>
+      <c r="CQ72" t="n">
+        <v>0.02607572967595826</v>
+      </c>
+      <c r="CR72" t="n">
+        <v>0.1593605534560689</v>
+      </c>
+      <c r="CS72" t="n">
+        <v>0.02607572967595826</v>
+      </c>
+      <c r="CT72" t="n">
+        <v>0.1593605534560689</v>
+      </c>
+      <c r="CU72" t="n">
+        <v>0.9739242703240417</v>
+      </c>
+      <c r="CV72" t="n">
+        <v>37.3498376620345</v>
+      </c>
+      <c r="CW72" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -20066,6 +23554,54 @@
       <c r="CG73" t="n">
         <v>0.3537918871252205</v>
       </c>
+      <c r="CH73" t="n">
+        <v>0.03135755570310544</v>
+      </c>
+      <c r="CI73" t="n">
+        <v>0.1309518122290148</v>
+      </c>
+      <c r="CJ73" t="n">
+        <v>0.1995409287174577</v>
+      </c>
+      <c r="CK73" t="n">
+        <v>1407093.312635554</v>
+      </c>
+      <c r="CL73" t="n">
+        <v>0.332280403353177</v>
+      </c>
+      <c r="CM73" t="n">
+        <v>0.4451290417758648</v>
+      </c>
+      <c r="CN73" t="n">
+        <v>5</v>
+      </c>
+      <c r="CO73" t="n">
+        <v>97.2619057157312</v>
+      </c>
+      <c r="CP73" t="n">
+        <v>52.35023075667934</v>
+      </c>
+      <c r="CQ73" t="n">
+        <v>0.660759845184581</v>
+      </c>
+      <c r="CR73" t="n">
+        <v>0.47345144648235</v>
+      </c>
+      <c r="CS73" t="n">
+        <v>0.6898831941961574</v>
+      </c>
+      <c r="CT73" t="n">
+        <v>0.3574296031902431</v>
+      </c>
+      <c r="CU73" t="n">
+        <v>0.1354114237117517</v>
+      </c>
+      <c r="CV73" t="n">
+        <v>0.5134091565757366</v>
+      </c>
+      <c r="CW73" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -20333,6 +23869,54 @@
       <c r="CG74" t="n">
         <v>0.4545454545454545</v>
       </c>
+      <c r="CH74" t="n">
+        <v>0.1170429188753796</v>
+      </c>
+      <c r="CI74" t="n">
+        <v>0.2908138785969713</v>
+      </c>
+      <c r="CJ74" t="n">
+        <v>0.2374798127677064</v>
+      </c>
+      <c r="CK74" t="n">
+        <v>2528691.151608358</v>
+      </c>
+      <c r="CL74" t="n">
+        <v>-0.1142162310457228</v>
+      </c>
+      <c r="CM74" t="n">
+        <v>0.4487414964404786</v>
+      </c>
+      <c r="CN74" t="n">
+        <v>8</v>
+      </c>
+      <c r="CO74" t="n">
+        <v>81.5771254568586</v>
+      </c>
+      <c r="CP74" t="n">
+        <v>21.99423164635925</v>
+      </c>
+      <c r="CQ74" t="n">
+        <v>0.8313479682130784</v>
+      </c>
+      <c r="CR74" t="n">
+        <v>0.3166627495556293</v>
+      </c>
+      <c r="CS74" t="n">
+        <v>0.7587765104135183</v>
+      </c>
+      <c r="CT74" t="n">
+        <v>0.3306103375843131</v>
+      </c>
+      <c r="CU74" t="n">
+        <v>0.05888206382493943</v>
+      </c>
+      <c r="CV74" t="n">
+        <v>0.2600011717834392</v>
+      </c>
+      <c r="CW74" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -20600,6 +24184,54 @@
       <c r="CG75" t="n">
         <v>0.3568958893584326</v>
       </c>
+      <c r="CH75" t="n">
+        <v>0.02506775805205124</v>
+      </c>
+      <c r="CI75" t="n">
+        <v>0.1292779659657242</v>
+      </c>
+      <c r="CJ75" t="n">
+        <v>0.1571898628398057</v>
+      </c>
+      <c r="CK75" t="n">
+        <v>1847434.311567487</v>
+      </c>
+      <c r="CL75" t="n">
+        <v>0.8455492835432045</v>
+      </c>
+      <c r="CM75" t="n">
+        <v>0.4449848024316109</v>
+      </c>
+      <c r="CN75" t="n">
+        <v>2</v>
+      </c>
+      <c r="CO75" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP75" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ75" t="n">
+        <v>0.02042987407729049</v>
+      </c>
+      <c r="CR75" t="n">
+        <v>0.1414655234411429</v>
+      </c>
+      <c r="CS75" t="n">
+        <v>0.008171949630916197</v>
+      </c>
+      <c r="CT75" t="n">
+        <v>0.05658620937645715</v>
+      </c>
+      <c r="CU75" t="n">
+        <v>0.9795701259227095</v>
+      </c>
+      <c r="CV75" t="n">
+        <v>4606000000000</v>
+      </c>
+      <c r="CW75" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -20866,6 +24498,54 @@
       </c>
       <c r="CG76" t="n">
         <v>0.3226256983240224</v>
+      </c>
+      <c r="CH76" t="n">
+        <v>0.0155522417302522</v>
+      </c>
+      <c r="CI76" t="n">
+        <v>0.201762513962105</v>
+      </c>
+      <c r="CJ76" t="n">
+        <v>0.24185753101099</v>
+      </c>
+      <c r="CK76" t="n">
+        <v>1883878.563222351</v>
+      </c>
+      <c r="CL76" t="n">
+        <v>-0.323488241881299</v>
+      </c>
+      <c r="CM76" t="n">
+        <v>-0.5318449048152296</v>
+      </c>
+      <c r="CN76" t="n">
+        <v>2</v>
+      </c>
+      <c r="CO76" t="n">
+        <v>179.618837938833</v>
+      </c>
+      <c r="CP76" t="n">
+        <v>11.88605864480795</v>
+      </c>
+      <c r="CQ76" t="n">
+        <v>0.01298292273236282</v>
+      </c>
+      <c r="CR76" t="n">
+        <v>0.1132005585219805</v>
+      </c>
+      <c r="CS76" t="n">
+        <v>0.01298292273236282</v>
+      </c>
+      <c r="CT76" t="n">
+        <v>0.1132005585219805</v>
+      </c>
+      <c r="CU76" t="n">
+        <v>0.9870170772676372</v>
+      </c>
+      <c r="CV76" t="n">
+        <v>76.02425875805865</v>
+      </c>
+      <c r="CW76" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>